<commit_message>
Actualización completa: Diseño de goleadores y tablas
</commit_message>
<xml_diff>
--- a/CAMPEONATO CACMQ 2026 (1).xlsx
+++ b/CAMPEONATO CACMQ 2026 (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\CACMQ\JORNADAS DEPORTIVAS 2026 MAYO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4DF84E-6E05-4193-B1F6-5A4645550CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8792F397-3A15-40D8-A9A5-07CDBE8669F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MASTER" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="88">
   <si>
     <t>N</t>
   </si>
@@ -295,6 +295,12 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>05 DE JUNIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GALLOS </t>
   </si>
 </sst>
 </file>
@@ -417,22 +423,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1698,34 +1704,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="15" t="s">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="I1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
       <c r="M1" s="4" t="s">
@@ -1748,34 +1754,34 @@
       </c>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="11">
-        <v>1</v>
-      </c>
-      <c r="B2" s="11" t="s">
+      <c r="A2" s="10">
+        <v>1</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="11">
-        <v>3</v>
-      </c>
-      <c r="D2" s="11">
-        <v>3</v>
-      </c>
-      <c r="E2" s="11">
-        <v>0</v>
-      </c>
-      <c r="F2" s="11">
-        <v>0</v>
-      </c>
-      <c r="G2" s="11">
+      <c r="C2" s="10">
+        <v>3</v>
+      </c>
+      <c r="D2" s="10">
+        <v>3</v>
+      </c>
+      <c r="E2" s="10">
+        <v>0</v>
+      </c>
+      <c r="F2" s="10">
+        <v>0</v>
+      </c>
+      <c r="G2" s="10">
         <v>15</v>
       </c>
-      <c r="H2" s="11">
-        <v>2</v>
-      </c>
-      <c r="I2" s="11">
+      <c r="H2" s="10">
+        <v>2</v>
+      </c>
+      <c r="I2" s="10">
         <v>13</v>
       </c>
-      <c r="J2" s="11">
+      <c r="J2" s="10">
         <v>9</v>
       </c>
       <c r="T2" s="4" t="s">
@@ -1789,42 +1795,42 @@
       </c>
     </row>
     <row r="3" spans="1:22">
-      <c r="A3" s="11">
-        <v>2</v>
-      </c>
-      <c r="B3" s="11" t="s">
+      <c r="A3" s="10">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="11">
-        <v>4</v>
-      </c>
-      <c r="D3" s="11">
-        <v>2</v>
-      </c>
-      <c r="E3" s="11">
-        <v>1</v>
-      </c>
-      <c r="F3" s="11">
-        <v>1</v>
-      </c>
-      <c r="G3" s="11">
+      <c r="C3" s="10">
+        <v>4</v>
+      </c>
+      <c r="D3" s="10">
+        <v>2</v>
+      </c>
+      <c r="E3" s="10">
+        <v>1</v>
+      </c>
+      <c r="F3" s="10">
+        <v>1</v>
+      </c>
+      <c r="G3" s="10">
         <v>12</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3" s="10">
         <v>7</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="10">
         <v>5</v>
       </c>
-      <c r="J3" s="11">
+      <c r="J3" s="10">
         <v>7</v>
       </c>
-      <c r="M3" s="10" t="s">
+      <c r="M3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
       <c r="T3" s="4" t="s">
         <v>41</v>
       </c>
@@ -1836,46 +1842,46 @@
       </c>
     </row>
     <row r="4" spans="1:22">
-      <c r="A4" s="11">
-        <v>3</v>
-      </c>
-      <c r="B4" s="11" t="s">
+      <c r="A4" s="10">
+        <v>3</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="11">
-        <v>3</v>
-      </c>
-      <c r="D4" s="11">
-        <v>2</v>
-      </c>
-      <c r="E4" s="11">
-        <v>1</v>
-      </c>
-      <c r="F4" s="11">
-        <v>0</v>
-      </c>
-      <c r="G4" s="11">
+      <c r="C4" s="10">
+        <v>3</v>
+      </c>
+      <c r="D4" s="10">
+        <v>2</v>
+      </c>
+      <c r="E4" s="10">
+        <v>1</v>
+      </c>
+      <c r="F4" s="10">
+        <v>0</v>
+      </c>
+      <c r="G4" s="10">
         <v>11</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <v>9</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="10">
         <v>8</v>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="10">
         <v>7</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="M4" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="N4" s="11">
-        <v>4</v>
-      </c>
-      <c r="O4" s="11">
-        <v>4</v>
-      </c>
-      <c r="P4" s="11" t="s">
+      <c r="N4" s="10">
+        <v>4</v>
+      </c>
+      <c r="O4" s="10">
+        <v>4</v>
+      </c>
+      <c r="P4" s="10" t="s">
         <v>45</v>
       </c>
       <c r="T4" s="4" t="s">
@@ -1889,372 +1895,372 @@
       </c>
     </row>
     <row r="5" spans="1:22">
-      <c r="A5" s="11">
-        <v>4</v>
-      </c>
-      <c r="B5" s="11" t="s">
+      <c r="A5" s="10">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="11">
-        <v>4</v>
-      </c>
-      <c r="D5" s="11">
-        <v>2</v>
-      </c>
-      <c r="E5" s="11">
-        <v>1</v>
-      </c>
-      <c r="F5" s="11">
-        <v>1</v>
-      </c>
-      <c r="G5" s="11">
+      <c r="C5" s="10">
+        <v>4</v>
+      </c>
+      <c r="D5" s="10">
+        <v>2</v>
+      </c>
+      <c r="E5" s="10">
+        <v>1</v>
+      </c>
+      <c r="F5" s="10">
+        <v>1</v>
+      </c>
+      <c r="G5" s="10">
         <v>13</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="10">
         <v>13</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="10">
         <v>6</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="10">
         <v>7</v>
       </c>
-      <c r="M5" s="10" t="s">
+      <c r="M5" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="N5" s="10"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
     </row>
     <row r="6" spans="1:22">
-      <c r="A6" s="11">
+      <c r="A6" s="10">
         <v>5</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="11">
-        <v>4</v>
-      </c>
-      <c r="D6" s="11">
-        <v>0</v>
-      </c>
-      <c r="E6" s="11">
-        <v>2</v>
-      </c>
-      <c r="F6" s="11">
-        <v>2</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="C6" s="10">
+        <v>4</v>
+      </c>
+      <c r="D6" s="10">
+        <v>0</v>
+      </c>
+      <c r="E6" s="10">
+        <v>2</v>
+      </c>
+      <c r="F6" s="10">
+        <v>2</v>
+      </c>
+      <c r="G6" s="10">
         <v>8</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <v>14</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="10">
         <v>-6</v>
       </c>
-      <c r="J6" s="11">
-        <v>2</v>
-      </c>
-      <c r="M6" s="11" t="s">
+      <c r="J6" s="10">
+        <v>2</v>
+      </c>
+      <c r="M6" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="N6" s="11">
-        <v>3</v>
-      </c>
-      <c r="O6" s="11">
+      <c r="N6" s="10">
+        <v>3</v>
+      </c>
+      <c r="O6" s="10">
         <v>6</v>
       </c>
-      <c r="P6" s="11" t="s">
+      <c r="P6" s="10" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:22">
-      <c r="A7" s="11">
+      <c r="A7" s="10">
         <v>6</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="11">
-        <v>3</v>
-      </c>
-      <c r="D7" s="11">
-        <v>0</v>
-      </c>
-      <c r="E7" s="11">
-        <v>1</v>
-      </c>
-      <c r="F7" s="11">
-        <v>2</v>
-      </c>
-      <c r="G7" s="11">
-        <v>4</v>
-      </c>
-      <c r="H7" s="11">
+      <c r="C7" s="10">
+        <v>3</v>
+      </c>
+      <c r="D7" s="10">
+        <v>0</v>
+      </c>
+      <c r="E7" s="10">
+        <v>1</v>
+      </c>
+      <c r="F7" s="10">
+        <v>2</v>
+      </c>
+      <c r="G7" s="10">
+        <v>4</v>
+      </c>
+      <c r="H7" s="10">
         <v>10</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="10">
         <v>-6</v>
       </c>
-      <c r="J7" s="11">
-        <v>1</v>
-      </c>
-      <c r="M7" s="10" t="s">
+      <c r="J7" s="10">
+        <v>1</v>
+      </c>
+      <c r="M7" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
     </row>
     <row r="8" spans="1:22">
-      <c r="A8" s="11">
+      <c r="A8" s="10">
         <v>7</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="11">
-        <v>3</v>
-      </c>
-      <c r="D8" s="11">
-        <v>0</v>
-      </c>
-      <c r="E8" s="11">
-        <v>0</v>
-      </c>
-      <c r="F8" s="11">
-        <v>3</v>
-      </c>
-      <c r="G8" s="11">
-        <v>4</v>
-      </c>
-      <c r="H8" s="11">
+      <c r="C8" s="10">
+        <v>3</v>
+      </c>
+      <c r="D8" s="10">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10">
+        <v>0</v>
+      </c>
+      <c r="F8" s="10">
+        <v>3</v>
+      </c>
+      <c r="G8" s="10">
+        <v>4</v>
+      </c>
+      <c r="H8" s="10">
         <v>19</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="10">
         <v>-15</v>
       </c>
-      <c r="J8" s="11">
-        <v>0</v>
-      </c>
-      <c r="M8" s="11" t="s">
+      <c r="J8" s="10">
+        <v>0</v>
+      </c>
+      <c r="M8" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="N8" s="11">
-        <v>3</v>
-      </c>
-      <c r="O8" s="11">
-        <v>2</v>
-      </c>
-      <c r="P8" s="11" t="s">
+      <c r="N8" s="10">
+        <v>3</v>
+      </c>
+      <c r="O8" s="10">
+        <v>2</v>
+      </c>
+      <c r="P8" s="10" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:22">
-      <c r="M9" s="10" t="s">
+      <c r="M9" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="13"/>
     </row>
     <row r="10" spans="1:22">
-      <c r="M10" s="11" t="s">
+      <c r="M10" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="N10" s="11">
-        <v>0</v>
-      </c>
-      <c r="O10" s="11">
-        <v>0</v>
-      </c>
-      <c r="P10" s="11" t="s">
+      <c r="N10" s="10">
+        <v>0</v>
+      </c>
+      <c r="O10" s="10">
+        <v>0</v>
+      </c>
+      <c r="P10" s="10" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:22">
-      <c r="M11" s="10" t="s">
+      <c r="M11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="10"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="13"/>
     </row>
     <row r="12" spans="1:22">
-      <c r="M12" s="11" t="s">
+      <c r="M12" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="N12" s="11">
+      <c r="N12" s="10">
         <v>5</v>
       </c>
-      <c r="O12" s="11">
+      <c r="O12" s="10">
         <v>6</v>
       </c>
-      <c r="P12" s="11" t="s">
+      <c r="P12" s="10" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:22">
-      <c r="M13" s="10" t="s">
+      <c r="M13" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="N13" s="10"/>
-      <c r="O13" s="10"/>
-      <c r="P13" s="10"/>
+      <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
+      <c r="P13" s="13"/>
     </row>
     <row r="14" spans="1:22">
-      <c r="M14" s="11" t="s">
+      <c r="M14" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="N14" s="11">
-        <v>0</v>
-      </c>
-      <c r="O14" s="11">
+      <c r="N14" s="10">
+        <v>0</v>
+      </c>
+      <c r="O14" s="10">
         <v>9</v>
       </c>
-      <c r="P14" s="11" t="s">
+      <c r="P14" s="10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:22">
-      <c r="M15" s="10" t="s">
+      <c r="M15" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
+      <c r="N15" s="13"/>
+      <c r="O15" s="13"/>
+      <c r="P15" s="13"/>
     </row>
     <row r="16" spans="1:22">
-      <c r="M16" s="11" t="s">
+      <c r="M16" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="N16" s="11">
+      <c r="N16" s="10">
         <v>5</v>
       </c>
-      <c r="O16" s="11">
-        <v>3</v>
-      </c>
-      <c r="P16" s="11" t="s">
+      <c r="O16" s="10">
+        <v>3</v>
+      </c>
+      <c r="P16" s="10" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="17" spans="13:16">
-      <c r="M17" s="12" t="s">
+      <c r="M17" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="N17" s="12"/>
-      <c r="O17" s="12"/>
-      <c r="P17" s="12"/>
+      <c r="N17" s="14"/>
+      <c r="O17" s="14"/>
+      <c r="P17" s="14"/>
     </row>
     <row r="18" spans="13:16">
-      <c r="M18" s="11" t="s">
+      <c r="M18" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="N18" s="11">
+      <c r="N18" s="10">
         <v>5</v>
       </c>
-      <c r="O18" s="11">
-        <v>1</v>
-      </c>
-      <c r="P18" s="11" t="s">
+      <c r="O18" s="10">
+        <v>1</v>
+      </c>
+      <c r="P18" s="10" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="19" spans="13:16">
-      <c r="M19" s="11" t="s">
+      <c r="M19" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="N19" s="11">
-        <v>0</v>
-      </c>
-      <c r="O19" s="11">
-        <v>3</v>
-      </c>
-      <c r="P19" s="11" t="s">
+      <c r="N19" s="10">
+        <v>0</v>
+      </c>
+      <c r="O19" s="10">
+        <v>3</v>
+      </c>
+      <c r="P19" s="10" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="20" spans="13:16">
-      <c r="M20" s="12" t="s">
+      <c r="M20" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="N20" s="12"/>
-      <c r="O20" s="12"/>
-      <c r="P20" s="12"/>
+      <c r="N20" s="14"/>
+      <c r="O20" s="14"/>
+      <c r="P20" s="14"/>
     </row>
     <row r="21" spans="13:16">
-      <c r="M21" s="11" t="s">
+      <c r="M21" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="N21" s="11">
-        <v>0</v>
-      </c>
-      <c r="O21" s="11">
-        <v>3</v>
-      </c>
-      <c r="P21" s="11" t="s">
+      <c r="N21" s="10">
+        <v>0</v>
+      </c>
+      <c r="O21" s="10">
+        <v>3</v>
+      </c>
+      <c r="P21" s="10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="22" spans="13:16">
-      <c r="M22" s="12" t="s">
+      <c r="M22" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="N22" s="12"/>
-      <c r="O22" s="12"/>
-      <c r="P22" s="12"/>
+      <c r="N22" s="14"/>
+      <c r="O22" s="14"/>
+      <c r="P22" s="14"/>
     </row>
     <row r="23" spans="13:16">
-      <c r="M23" s="11" t="s">
+      <c r="M23" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="N23" s="11">
-        <v>1</v>
-      </c>
-      <c r="O23" s="11">
-        <v>4</v>
-      </c>
-      <c r="P23" s="11" t="s">
+      <c r="N23" s="10">
+        <v>1</v>
+      </c>
+      <c r="O23" s="10">
+        <v>4</v>
+      </c>
+      <c r="P23" s="10" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="24" spans="13:16">
-      <c r="M24" s="13" t="s">
+      <c r="M24" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="N24" s="12"/>
-      <c r="O24" s="12"/>
-      <c r="P24" s="12"/>
+      <c r="N24" s="14"/>
+      <c r="O24" s="14"/>
+      <c r="P24" s="14"/>
     </row>
     <row r="25" spans="13:16">
-      <c r="M25" s="14" t="s">
+      <c r="M25" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="N25" s="11">
-        <v>3</v>
-      </c>
-      <c r="O25" s="11">
-        <v>3</v>
-      </c>
-      <c r="P25" s="14" t="s">
+      <c r="N25" s="10">
+        <v>3</v>
+      </c>
+      <c r="O25" s="10">
+        <v>3</v>
+      </c>
+      <c r="P25" s="11" t="s">
         <v>42</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="M13:P13"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="M5:P5"/>
+    <mergeCell ref="M7:P7"/>
+    <mergeCell ref="M9:P9"/>
+    <mergeCell ref="M11:P11"/>
     <mergeCell ref="M15:P15"/>
     <mergeCell ref="M17:P17"/>
     <mergeCell ref="M20:P20"/>
     <mergeCell ref="M22:P22"/>
     <mergeCell ref="M24:P24"/>
-    <mergeCell ref="M3:P3"/>
-    <mergeCell ref="M5:P5"/>
-    <mergeCell ref="M7:P7"/>
-    <mergeCell ref="M9:P9"/>
-    <mergeCell ref="M11:P11"/>
-    <mergeCell ref="M13:P13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3396,7 +3402,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="27.33203125" customWidth="1"/>
@@ -3440,16 +3446,16 @@
         <v>73</v>
       </c>
       <c r="C2" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" s="4">
         <v>0</v>
       </c>
       <c r="F2" s="4">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
@@ -3461,7 +3467,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C3" s="4">
         <v>5</v>
@@ -3473,7 +3479,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>47</v>
@@ -3487,19 +3493,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C4" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" s="4">
         <v>1</v>
       </c>
       <c r="F4" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>75</v>
@@ -3523,13 +3529,13 @@
         <v>77</v>
       </c>
       <c r="C5" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="4">
         <v>3</v>
       </c>
       <c r="E5" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="4">
         <v>9</v>
@@ -3555,7 +3561,7 @@
         <v>76</v>
       </c>
       <c r="C6" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" s="4">
         <v>1</v>
@@ -3564,7 +3570,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="4">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>79</v>
@@ -3587,7 +3593,7 @@
         <v>78</v>
       </c>
       <c r="C7" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" s="4">
         <v>1</v>
@@ -3616,19 +3622,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="C8" s="4">
         <v>4</v>
       </c>
       <c r="D8" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>80</v>
@@ -3642,16 +3648,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="C9" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D9" s="4">
         <v>0</v>
       </c>
       <c r="E9" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F9" s="4">
         <v>1</v>
@@ -3677,13 +3683,13 @@
         <v>79</v>
       </c>
       <c r="C10" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="4">
         <v>0</v>
       </c>
       <c r="E10" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" s="4">
         <v>0</v>
@@ -3906,6 +3912,70 @@
         <v>74</v>
       </c>
     </row>
+    <row r="25" spans="1:12">
+      <c r="I25" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="I26" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J26" s="4">
+        <v>3</v>
+      </c>
+      <c r="K26" s="4">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="I27" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="J27" s="4">
+        <v>1</v>
+      </c>
+      <c r="K27" s="4">
+        <v>2</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="I28" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J28" s="4">
+        <v>0</v>
+      </c>
+      <c r="K28" s="4">
+        <v>3</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="I29" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="J29" s="4">
+        <v>0</v>
+      </c>
+      <c r="K29" s="4">
+        <v>3</v>
+      </c>
+      <c r="L29" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización: Cambios en diseño y datos de fútbol
</commit_message>
<xml_diff>
--- a/CAMPEONATO CACMQ 2026 (1).xlsx
+++ b/CAMPEONATO CACMQ 2026 (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\CACMQ\JORNADAS DEPORTIVAS 2026 MAYO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8792F397-3A15-40D8-A9A5-07CDBE8669F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADCAEB5-4165-4E6E-A37E-B77366EB379E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MASTER" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="93">
   <si>
     <t>N</t>
   </si>
@@ -177,9 +177,6 @@
     <t>GAT-S 1</t>
   </si>
   <si>
-    <t>ANGEL PERDOMO</t>
-  </si>
-  <si>
     <t>19 DE MAYO</t>
   </si>
   <si>
@@ -301,18 +298,43 @@
   </si>
   <si>
     <t xml:space="preserve">GALLOS </t>
+  </si>
+  <si>
+    <t>08 DE JUNIO</t>
+  </si>
+  <si>
+    <t>GABRIEL PUENTE</t>
+  </si>
+  <si>
+    <t>JIMMY PENALOZA</t>
+  </si>
+  <si>
+    <t>SEBASTIAN CHIMBORAZO</t>
+  </si>
+  <si>
+    <t>JOSE SANTACRUZ</t>
+  </si>
+  <si>
+    <t>8 DE JUNIO  /DIFERIDO/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -330,8 +352,16 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -352,13 +382,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39994506668294322"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -392,23 +416,23 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -417,28 +441,31 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -936,7 +963,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W31"/>
+  <dimension ref="A1:W35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="4" customWidth="1"/>
@@ -1000,55 +1027,46 @@
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
-      <c r="U1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="2" spans="1:23">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C2" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E2" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" s="4">
         <v>0</v>
       </c>
       <c r="G2" s="4">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="H2" s="4">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I2" s="4">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J2" s="4">
+        <v>18</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W2" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="U2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="V2" s="4">
-        <v>7</v>
-      </c>
-      <c r="W2" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -1056,10 +1074,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="4">
         <v>5</v>
@@ -1068,16 +1086,16 @@
         <v>0</v>
       </c>
       <c r="F3" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="4">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H3" s="4">
         <v>7</v>
       </c>
       <c r="I3" s="4">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="J3" s="4">
         <v>15</v>
@@ -1089,10 +1107,10 @@
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="U3" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="V3" s="4">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="W3" s="4" t="s">
         <v>16</v>
@@ -1103,7 +1121,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" s="4">
         <v>5</v>
@@ -1112,22 +1130,22 @@
         <v>4</v>
       </c>
       <c r="E4" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="4">
         <v>17</v>
       </c>
       <c r="H4" s="4">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I4" s="4">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="J4" s="4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M4" s="4" t="s">
         <v>20</v>
@@ -1142,13 +1160,13 @@
         <v>21</v>
       </c>
       <c r="U4" s="4" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="V4" s="4">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="W4" s="4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:23">
@@ -1156,7 +1174,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C5" s="4">
         <v>5</v>
@@ -1171,13 +1189,13 @@
         <v>2</v>
       </c>
       <c r="G5" s="4">
+        <v>13</v>
+      </c>
+      <c r="H5" s="4">
+        <v>8</v>
+      </c>
+      <c r="I5" s="4">
         <v>5</v>
-      </c>
-      <c r="H5" s="4">
-        <v>12</v>
-      </c>
-      <c r="I5" s="4">
-        <v>-7</v>
       </c>
       <c r="J5" s="4">
         <v>7</v>
@@ -1188,19 +1206,28 @@
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
+      <c r="U5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="V5" s="4">
+        <v>6</v>
+      </c>
+      <c r="W5" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="6" spans="1:23">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C6" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="4">
         <v>1</v>
@@ -1209,16 +1236,16 @@
         <v>2</v>
       </c>
       <c r="G6" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H6" s="4">
+        <v>12</v>
+      </c>
+      <c r="I6" s="4">
+        <v>-7</v>
+      </c>
+      <c r="J6" s="4">
         <v>7</v>
-      </c>
-      <c r="I6" s="4">
-        <v>3</v>
-      </c>
-      <c r="J6" s="4">
-        <v>4</v>
       </c>
       <c r="M6" s="4" t="s">
         <v>26</v>
@@ -1231,6 +1258,15 @@
       </c>
       <c r="P6" s="4" t="s">
         <v>27</v>
+      </c>
+      <c r="U6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="V6" s="4">
+        <v>4</v>
+      </c>
+      <c r="W6" s="4" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:23">
@@ -1238,10 +1274,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="4">
         <v>1</v>
@@ -1250,16 +1286,16 @@
         <v>1</v>
       </c>
       <c r="F7" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G7" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H7" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I7" s="4">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="J7" s="4">
         <v>4</v>
@@ -1282,7 +1318,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" s="4">
         <v>5</v>
@@ -1297,13 +1333,13 @@
         <v>3</v>
       </c>
       <c r="G8" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H8" s="4">
         <v>15</v>
       </c>
       <c r="I8" s="4">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="J8" s="4">
         <v>4</v>
@@ -1326,7 +1362,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C9" s="4">
         <v>6</v>
@@ -1344,10 +1380,10 @@
         <v>7</v>
       </c>
       <c r="H9" s="4">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I9" s="4">
-        <v>-7</v>
+        <v>-11</v>
       </c>
       <c r="J9" s="4">
         <v>4</v>
@@ -1373,7 +1409,7 @@
         <v>31</v>
       </c>
       <c r="C10" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10" s="4">
         <v>0</v>
@@ -1382,16 +1418,16 @@
         <v>0</v>
       </c>
       <c r="F10" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G10" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H10" s="4">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="I10" s="4">
-        <v>-11</v>
+        <v>-20</v>
       </c>
       <c r="J10" s="4">
         <v>0</v>
@@ -1625,23 +1661,23 @@
     </row>
     <row r="28" spans="13:17">
       <c r="M28" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
       <c r="P28" s="6"/>
     </row>
     <row r="29" spans="13:17">
-      <c r="M29" s="9" t="s">
+      <c r="M29" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="N29" s="9">
-        <v>1</v>
-      </c>
-      <c r="O29" s="9">
-        <v>0</v>
-      </c>
-      <c r="P29" s="9" t="s">
+      <c r="N29" s="8">
+        <v>1</v>
+      </c>
+      <c r="O29" s="8">
+        <v>0</v>
+      </c>
+      <c r="P29" s="8" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1655,11 +1691,11 @@
       <c r="O30" s="4">
         <v>5</v>
       </c>
-      <c r="P30" s="9" t="s">
+      <c r="P30" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="Q30" s="9" t="s">
-        <v>85</v>
+      <c r="Q30" s="8" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="31" spans="13:17">
@@ -1674,6 +1710,56 @@
       </c>
       <c r="P31" s="4" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="13:17">
+      <c r="M32" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="N32" s="6"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="6"/>
+    </row>
+    <row r="33" spans="13:16">
+      <c r="M33" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N33" s="8">
+        <v>10</v>
+      </c>
+      <c r="O33" s="8">
+        <v>1</v>
+      </c>
+      <c r="P33" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="13:16">
+      <c r="M34" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="N34" s="4">
+        <v>3</v>
+      </c>
+      <c r="O34" s="4">
+        <v>1</v>
+      </c>
+      <c r="P34" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="13:16">
+      <c r="M35" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="N35" s="4">
+        <v>6</v>
+      </c>
+      <c r="O35" s="4">
+        <v>2</v>
+      </c>
+      <c r="P35" s="4" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1683,7 +1769,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:V25"/>
+  <dimension ref="A1:V27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="27.88671875" style="4" customWidth="1"/>
@@ -1698,564 +1784,601 @@
     <col min="14" max="14" width="5.33203125" style="4" customWidth="1"/>
     <col min="15" max="15" width="5.6640625" style="4" customWidth="1"/>
     <col min="16" max="16" width="26.77734375" style="4" customWidth="1"/>
-    <col min="20" max="20" width="22.77734375" style="4" customWidth="1"/>
+    <col min="19" max="19" width="7.44140625" customWidth="1"/>
+    <col min="20" max="20" width="25.21875" style="4" customWidth="1"/>
     <col min="21" max="21" width="9.109375" style="4"/>
     <col min="22" max="22" width="18.33203125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
-      <c r="A1" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="12" t="s">
+    <row r="1" spans="1:22" s="14" customFormat="1">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="P1" s="15"/>
+      <c r="T1" s="15"/>
+      <c r="U1" s="15"/>
+      <c r="V1" s="15"/>
+    </row>
+    <row r="2" spans="1:22">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="9">
+        <v>5</v>
+      </c>
+      <c r="D2" s="9">
+        <v>3</v>
+      </c>
+      <c r="E2" s="9">
+        <v>1</v>
+      </c>
+      <c r="F2" s="9">
+        <v>1</v>
+      </c>
+      <c r="G2" s="9">
+        <v>20</v>
+      </c>
+      <c r="H2" s="9">
+        <v>16</v>
+      </c>
+      <c r="I2" s="9">
+        <v>4</v>
+      </c>
+      <c r="J2" s="9">
+        <v>10</v>
+      </c>
+      <c r="T2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="U2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="V1" s="8" t="s">
+      <c r="V2" s="15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:22">
-      <c r="A2" s="10">
-        <v>1</v>
-      </c>
-      <c r="B2" s="10" t="s">
+    <row r="3" spans="1:22">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="10">
-        <v>3</v>
-      </c>
-      <c r="D2" s="10">
-        <v>3</v>
-      </c>
-      <c r="E2" s="10">
-        <v>0</v>
-      </c>
-      <c r="F2" s="10">
-        <v>0</v>
-      </c>
-      <c r="G2" s="10">
+      <c r="C3" s="9">
+        <v>3</v>
+      </c>
+      <c r="D3" s="9">
+        <v>3</v>
+      </c>
+      <c r="E3" s="9">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9">
+        <v>0</v>
+      </c>
+      <c r="G3" s="9">
         <v>15</v>
       </c>
-      <c r="H2" s="10">
-        <v>2</v>
-      </c>
-      <c r="I2" s="10">
+      <c r="H3" s="9">
+        <v>2</v>
+      </c>
+      <c r="I3" s="9">
         <v>13</v>
       </c>
-      <c r="J2" s="10">
+      <c r="J3" s="9">
         <v>9</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="M3" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="T3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="U2" s="4">
+      <c r="U3" s="4">
         <v>11</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="V3" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:22">
-      <c r="A3" s="10">
-        <v>2</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="10">
-        <v>4</v>
-      </c>
-      <c r="D3" s="10">
-        <v>2</v>
-      </c>
-      <c r="E3" s="10">
-        <v>1</v>
-      </c>
-      <c r="F3" s="10">
-        <v>1</v>
-      </c>
-      <c r="G3" s="10">
-        <v>12</v>
-      </c>
-      <c r="H3" s="10">
+    <row r="4" spans="1:22">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="9">
+        <v>3</v>
+      </c>
+      <c r="D4" s="9">
+        <v>2</v>
+      </c>
+      <c r="E4" s="9">
+        <v>1</v>
+      </c>
+      <c r="F4" s="9">
+        <v>0</v>
+      </c>
+      <c r="G4" s="9">
+        <v>11</v>
+      </c>
+      <c r="H4" s="9">
+        <v>9</v>
+      </c>
+      <c r="I4" s="9">
+        <v>8</v>
+      </c>
+      <c r="J4" s="9">
         <v>7</v>
       </c>
-      <c r="I3" s="10">
-        <v>5</v>
-      </c>
-      <c r="J3" s="10">
+      <c r="M4" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="N4" s="9">
+        <v>4</v>
+      </c>
+      <c r="O4" s="9">
+        <v>4</v>
+      </c>
+      <c r="P4" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="T4" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="U4" s="4">
         <v>7</v>
-      </c>
-      <c r="M3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="T3" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="U3" s="4">
-        <v>4</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22">
-      <c r="A4" s="10">
-        <v>3</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" s="10">
-        <v>3</v>
-      </c>
-      <c r="D4" s="10">
-        <v>2</v>
-      </c>
-      <c r="E4" s="10">
-        <v>1</v>
-      </c>
-      <c r="F4" s="10">
-        <v>0</v>
-      </c>
-      <c r="G4" s="10">
-        <v>11</v>
-      </c>
-      <c r="H4" s="10">
-        <v>9</v>
-      </c>
-      <c r="I4" s="10">
-        <v>8</v>
-      </c>
-      <c r="J4" s="10">
-        <v>7</v>
-      </c>
-      <c r="M4" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="N4" s="10">
-        <v>4</v>
-      </c>
-      <c r="O4" s="10">
-        <v>4</v>
-      </c>
-      <c r="P4" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="T4" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="U4" s="4">
-        <v>3</v>
       </c>
       <c r="V4" s="4" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:22">
-      <c r="A5" s="10">
-        <v>4</v>
-      </c>
-      <c r="B5" s="10" t="s">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="9">
+        <v>4</v>
+      </c>
+      <c r="D5" s="9">
+        <v>2</v>
+      </c>
+      <c r="E5" s="9">
+        <v>1</v>
+      </c>
+      <c r="F5" s="9">
+        <v>1</v>
+      </c>
+      <c r="G5" s="9">
+        <v>12</v>
+      </c>
+      <c r="H5" s="9">
+        <v>7</v>
+      </c>
+      <c r="I5" s="9">
+        <v>5</v>
+      </c>
+      <c r="J5" s="9">
+        <v>7</v>
+      </c>
+      <c r="M5" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="T5" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="U5" s="4">
+        <v>7</v>
+      </c>
+      <c r="V5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="10">
-        <v>4</v>
-      </c>
-      <c r="D5" s="10">
-        <v>2</v>
-      </c>
-      <c r="E5" s="10">
-        <v>1</v>
-      </c>
-      <c r="F5" s="10">
-        <v>1</v>
-      </c>
-      <c r="G5" s="10">
-        <v>13</v>
-      </c>
-      <c r="H5" s="10">
-        <v>13</v>
-      </c>
-      <c r="I5" s="10">
+    </row>
+    <row r="6" spans="1:22">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="9">
+        <v>4</v>
+      </c>
+      <c r="D6" s="9">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9">
+        <v>2</v>
+      </c>
+      <c r="F6" s="9">
+        <v>2</v>
+      </c>
+      <c r="G6" s="9">
+        <v>8</v>
+      </c>
+      <c r="H6" s="9">
+        <v>14</v>
+      </c>
+      <c r="I6" s="9">
+        <v>-6</v>
+      </c>
+      <c r="J6" s="9">
+        <v>2</v>
+      </c>
+      <c r="M6" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="N6" s="9">
+        <v>3</v>
+      </c>
+      <c r="O6" s="9">
         <v>6</v>
       </c>
-      <c r="J5" s="10">
+      <c r="P6" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="T6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="U6" s="4">
+        <v>6</v>
+      </c>
+      <c r="V6" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="9">
+        <v>4</v>
+      </c>
+      <c r="D7" s="9">
+        <v>0</v>
+      </c>
+      <c r="E7" s="9">
+        <v>1</v>
+      </c>
+      <c r="F7" s="9">
+        <v>3</v>
+      </c>
+      <c r="G7" s="9">
         <v>7</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="H7" s="9">
+        <v>17</v>
+      </c>
+      <c r="I7" s="9">
+        <v>-10</v>
+      </c>
+      <c r="J7" s="9">
+        <v>1</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+    </row>
+    <row r="8" spans="1:22">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-    </row>
-    <row r="6" spans="1:22">
-      <c r="A6" s="10">
+      <c r="C8" s="9">
+        <v>3</v>
+      </c>
+      <c r="D8" s="9">
+        <v>0</v>
+      </c>
+      <c r="E8" s="9">
+        <v>0</v>
+      </c>
+      <c r="F8" s="9">
+        <v>3</v>
+      </c>
+      <c r="G8" s="9">
+        <v>4</v>
+      </c>
+      <c r="H8" s="9">
+        <v>19</v>
+      </c>
+      <c r="I8" s="9">
+        <v>-15</v>
+      </c>
+      <c r="J8" s="9">
+        <v>0</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="N8" s="9">
+        <v>3</v>
+      </c>
+      <c r="O8" s="9">
+        <v>2</v>
+      </c>
+      <c r="P8" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22">
+      <c r="M9" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+    </row>
+    <row r="10" spans="1:22">
+      <c r="M10" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="N10" s="9">
+        <v>0</v>
+      </c>
+      <c r="O10" s="9">
+        <v>0</v>
+      </c>
+      <c r="P10" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22">
+      <c r="M11" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="N11" s="16"/>
+      <c r="O11" s="16"/>
+      <c r="P11" s="16"/>
+    </row>
+    <row r="12" spans="1:22">
+      <c r="M12" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="N12" s="9">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="O12" s="9">
+        <v>6</v>
+      </c>
+      <c r="P12" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
+      <c r="M13" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="N13" s="16"/>
+      <c r="O13" s="16"/>
+      <c r="P13" s="16"/>
+    </row>
+    <row r="14" spans="1:22">
+      <c r="M14" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="N14" s="9">
+        <v>0</v>
+      </c>
+      <c r="O14" s="9">
+        <v>9</v>
+      </c>
+      <c r="P14" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22">
+      <c r="M15" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N15" s="16"/>
+      <c r="O15" s="16"/>
+      <c r="P15" s="16"/>
+    </row>
+    <row r="16" spans="1:22">
+      <c r="M16" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="N16" s="9">
+        <v>5</v>
+      </c>
+      <c r="O16" s="9">
+        <v>3</v>
+      </c>
+      <c r="P16" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="10">
-        <v>4</v>
-      </c>
-      <c r="D6" s="10">
-        <v>0</v>
-      </c>
-      <c r="E6" s="10">
-        <v>2</v>
-      </c>
-      <c r="F6" s="10">
-        <v>2</v>
-      </c>
-      <c r="G6" s="10">
-        <v>8</v>
-      </c>
-      <c r="H6" s="10">
-        <v>14</v>
-      </c>
-      <c r="I6" s="10">
-        <v>-6</v>
-      </c>
-      <c r="J6" s="10">
-        <v>2</v>
-      </c>
-      <c r="M6" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="N6" s="10">
-        <v>3</v>
-      </c>
-      <c r="O6" s="10">
-        <v>6</v>
-      </c>
-      <c r="P6" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22">
-      <c r="A7" s="10">
-        <v>6</v>
-      </c>
-      <c r="B7" s="10" t="s">
+    </row>
+    <row r="17" spans="13:16">
+      <c r="M17" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="N17" s="16"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="16"/>
+    </row>
+    <row r="18" spans="13:16">
+      <c r="M18" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="N18" s="9">
+        <v>5</v>
+      </c>
+      <c r="O18" s="9">
+        <v>1</v>
+      </c>
+      <c r="P18" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="13:16">
+      <c r="M19" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="10">
-        <v>3</v>
-      </c>
-      <c r="D7" s="10">
-        <v>0</v>
-      </c>
-      <c r="E7" s="10">
-        <v>1</v>
-      </c>
-      <c r="F7" s="10">
-        <v>2</v>
-      </c>
-      <c r="G7" s="10">
-        <v>4</v>
-      </c>
-      <c r="H7" s="10">
-        <v>10</v>
-      </c>
-      <c r="I7" s="10">
-        <v>-6</v>
-      </c>
-      <c r="J7" s="10">
-        <v>1</v>
-      </c>
-      <c r="M7" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-    </row>
-    <row r="8" spans="1:22">
-      <c r="A8" s="10">
+      <c r="N19" s="9">
+        <v>0</v>
+      </c>
+      <c r="O19" s="9">
+        <v>3</v>
+      </c>
+      <c r="P19" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="13:16">
+      <c r="M20" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="16"/>
+    </row>
+    <row r="21" spans="13:16">
+      <c r="M21" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="N21" s="9">
+        <v>0</v>
+      </c>
+      <c r="O21" s="9">
+        <v>3</v>
+      </c>
+      <c r="P21" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="13:16">
+      <c r="M22" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16"/>
+    </row>
+    <row r="23" spans="13:16">
+      <c r="M23" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="N23" s="9">
+        <v>1</v>
+      </c>
+      <c r="O23" s="9">
+        <v>4</v>
+      </c>
+      <c r="P23" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="13:16">
+      <c r="M24" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="N24" s="16"/>
+      <c r="O24" s="16"/>
+      <c r="P24" s="16"/>
+    </row>
+    <row r="25" spans="13:16">
+      <c r="M25" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="N25" s="9">
+        <v>3</v>
+      </c>
+      <c r="O25" s="9">
+        <v>3</v>
+      </c>
+      <c r="P25" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="13:16">
+      <c r="M26" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="N26" s="16"/>
+      <c r="O26" s="16"/>
+      <c r="P26" s="16"/>
+    </row>
+    <row r="27" spans="13:16">
+      <c r="M27" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="N27" s="9">
+        <v>3</v>
+      </c>
+      <c r="O27" s="9">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="10">
-        <v>3</v>
-      </c>
-      <c r="D8" s="10">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10">
-        <v>0</v>
-      </c>
-      <c r="F8" s="10">
-        <v>3</v>
-      </c>
-      <c r="G8" s="10">
-        <v>4</v>
-      </c>
-      <c r="H8" s="10">
-        <v>19</v>
-      </c>
-      <c r="I8" s="10">
-        <v>-15</v>
-      </c>
-      <c r="J8" s="10">
-        <v>0</v>
-      </c>
-      <c r="M8" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="N8" s="10">
-        <v>3</v>
-      </c>
-      <c r="O8" s="10">
-        <v>2</v>
-      </c>
-      <c r="P8" s="10" t="s">
+      <c r="P27" s="10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:22">
-      <c r="M9" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
-    </row>
-    <row r="10" spans="1:22">
-      <c r="M10" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="N10" s="10">
-        <v>0</v>
-      </c>
-      <c r="O10" s="10">
-        <v>0</v>
-      </c>
-      <c r="P10" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22">
-      <c r="M11" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
-    </row>
-    <row r="12" spans="1:22">
-      <c r="M12" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="N12" s="10">
-        <v>5</v>
-      </c>
-      <c r="O12" s="10">
-        <v>6</v>
-      </c>
-      <c r="P12" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22">
-      <c r="M13" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="13"/>
-    </row>
-    <row r="14" spans="1:22">
-      <c r="M14" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="N14" s="10">
-        <v>0</v>
-      </c>
-      <c r="O14" s="10">
-        <v>9</v>
-      </c>
-      <c r="P14" s="10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22">
-      <c r="M15" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
-    </row>
-    <row r="16" spans="1:22">
-      <c r="M16" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="N16" s="10">
-        <v>5</v>
-      </c>
-      <c r="O16" s="10">
-        <v>3</v>
-      </c>
-      <c r="P16" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="17" spans="13:16">
-      <c r="M17" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="N17" s="14"/>
-      <c r="O17" s="14"/>
-      <c r="P17" s="14"/>
-    </row>
-    <row r="18" spans="13:16">
-      <c r="M18" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="N18" s="10">
-        <v>5</v>
-      </c>
-      <c r="O18" s="10">
-        <v>1</v>
-      </c>
-      <c r="P18" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="13:16">
-      <c r="M19" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="N19" s="10">
-        <v>0</v>
-      </c>
-      <c r="O19" s="10">
-        <v>3</v>
-      </c>
-      <c r="P19" s="10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="13:16">
-      <c r="M20" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="N20" s="14"/>
-      <c r="O20" s="14"/>
-      <c r="P20" s="14"/>
-    </row>
-    <row r="21" spans="13:16">
-      <c r="M21" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="N21" s="10">
-        <v>0</v>
-      </c>
-      <c r="O21" s="10">
-        <v>3</v>
-      </c>
-      <c r="P21" s="10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="22" spans="13:16">
-      <c r="M22" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="N22" s="14"/>
-      <c r="O22" s="14"/>
-      <c r="P22" s="14"/>
-    </row>
-    <row r="23" spans="13:16">
-      <c r="M23" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="N23" s="10">
-        <v>1</v>
-      </c>
-      <c r="O23" s="10">
-        <v>4</v>
-      </c>
-      <c r="P23" s="10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="24" spans="13:16">
-      <c r="M24" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="N24" s="14"/>
-      <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
-    </row>
-    <row r="25" spans="13:16">
-      <c r="M25" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="N25" s="10">
-        <v>3</v>
-      </c>
-      <c r="O25" s="10">
-        <v>3</v>
-      </c>
-      <c r="P25" s="11" t="s">
-        <v>42</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="M13:P13"/>
     <mergeCell ref="M3:P3"/>
     <mergeCell ref="M5:P5"/>
     <mergeCell ref="M7:P7"/>
     <mergeCell ref="M9:P9"/>
     <mergeCell ref="M11:P11"/>
+    <mergeCell ref="M26:P26"/>
     <mergeCell ref="M15:P15"/>
     <mergeCell ref="M17:P17"/>
     <mergeCell ref="M20:P20"/>
@@ -2284,7 +2407,7 @@
     <col min="14" max="14" width="5.109375" customWidth="1"/>
     <col min="15" max="15" width="4.88671875" customWidth="1"/>
     <col min="16" max="16" width="24.6640625" customWidth="1"/>
-    <col min="18" max="18" width="55.33203125" customWidth="1"/>
+    <col min="18" max="18" width="23.88671875" customWidth="1"/>
     <col min="20" max="20" width="27.5546875" customWidth="1"/>
     <col min="21" max="21" width="7.21875" customWidth="1"/>
     <col min="22" max="22" width="22.21875" customWidth="1"/>
@@ -2331,28 +2454,19 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="S1" s="1"/>
-      <c r="T1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="2" spans="1:22">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C2" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" s="4">
         <v>2</v>
@@ -2361,16 +2475,16 @@
         <v>1</v>
       </c>
       <c r="F2" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" s="4">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="H2" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I2" s="4">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="J2" s="4">
         <v>7</v>
@@ -2384,14 +2498,14 @@
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
-      <c r="T2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="U2" s="4">
+      <c r="T2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="U2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="V2" s="4" t="s">
-        <v>57</v>
+      <c r="V2" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -2399,13 +2513,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C3" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" s="4">
         <v>1</v>
@@ -2414,20 +2528,20 @@
         <v>1</v>
       </c>
       <c r="G3" s="4">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="H3" s="4">
+        <v>18</v>
+      </c>
+      <c r="I3" s="4">
+        <v>-9</v>
+      </c>
+      <c r="J3" s="4">
         <v>7</v>
-      </c>
-      <c r="I3" s="4">
-        <v>19</v>
-      </c>
-      <c r="J3" s="4">
-        <v>4</v>
       </c>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="6" t="s">
+      <c r="M3" s="11" t="s">
         <v>24</v>
       </c>
       <c r="N3" s="6"/>
@@ -2437,13 +2551,13 @@
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="U3" s="4">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -2451,7 +2565,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C4" s="4">
         <v>3</v>
@@ -2480,28 +2594,28 @@
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="N4" s="4">
+        <v>2</v>
+      </c>
+      <c r="O4" s="4">
+        <v>2</v>
+      </c>
+      <c r="P4" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="N4" s="4">
-        <v>2</v>
-      </c>
-      <c r="O4" s="4">
-        <v>2</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>60</v>
       </c>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4" t="s">
-        <v>61</v>
+        <v>91</v>
       </c>
       <c r="U4" s="4">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -2509,7 +2623,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="4">
         <v>3</v>
@@ -2537,8 +2651,8 @@
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
-      <c r="M5" s="6" t="s">
-        <v>47</v>
+      <c r="M5" s="12" t="s">
+        <v>46</v>
       </c>
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
@@ -2546,16 +2660,22 @@
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
+      <c r="T5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="U5" s="4">
+        <v>2</v>
+      </c>
+      <c r="V5" s="4" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="6" spans="1:22">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" s="4">
         <v>3</v>
@@ -2584,7 +2704,7 @@
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="N6" s="4">
         <v>4</v>
@@ -2593,21 +2713,27 @@
         <v>2</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
-      <c r="T6" s="4"/>
-      <c r="U6" s="4"/>
-      <c r="V6" s="4"/>
+      <c r="T6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U6" s="4">
+        <v>2</v>
+      </c>
+      <c r="V6" s="4" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="7" spans="1:22">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" s="4">
         <v>3</v>
@@ -2635,8 +2761,8 @@
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
-      <c r="M7" s="6" t="s">
-        <v>49</v>
+      <c r="M7" s="11" t="s">
+        <v>48</v>
       </c>
       <c r="N7" s="6"/>
       <c r="O7" s="6"/>
@@ -2662,7 +2788,7 @@
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N8" s="4">
         <v>12</v>
@@ -2671,7 +2797,7 @@
         <v>1</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
@@ -2682,18 +2808,9 @@
     </row>
     <row r="9" spans="1:22">
       <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
-      <c r="M9" s="6" t="s">
+      <c r="M9" s="11" t="s">
         <v>33</v>
       </c>
       <c r="N9" s="6"/>
@@ -2720,7 +2837,7 @@
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N10" s="4">
         <v>10</v>
@@ -2729,11 +2846,11 @@
         <v>2</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q10" s="4"/>
       <c r="R10" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
@@ -2744,8 +2861,8 @@
       <c r="A11" s="4"/>
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
-      <c r="M11" s="6" t="s">
-        <v>50</v>
+      <c r="M11" s="11" t="s">
+        <v>49</v>
       </c>
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
@@ -2762,7 +2879,7 @@
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N12" s="4">
         <v>3</v>
@@ -2771,7 +2888,7 @@
         <v>1</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
@@ -2784,8 +2901,8 @@
       <c r="A13" s="4"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="6" t="s">
-        <v>51</v>
+      <c r="M13" s="11" t="s">
+        <v>50</v>
       </c>
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
@@ -2802,7 +2919,7 @@
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N14" s="4">
         <v>1</v>
@@ -2811,7 +2928,7 @@
         <v>2</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
@@ -2833,8 +2950,8 @@
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="6" t="s">
-        <v>52</v>
+      <c r="M15" s="11" t="s">
+        <v>51</v>
       </c>
       <c r="N15" s="6"/>
       <c r="O15" s="6"/>
@@ -2860,7 +2977,7 @@
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="N16" s="4">
         <v>3</v>
@@ -2869,7 +2986,7 @@
         <v>3</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
@@ -2891,8 +3008,8 @@
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
-      <c r="M17" s="6" t="s">
-        <v>53</v>
+      <c r="M17" s="11" t="s">
+        <v>52</v>
       </c>
       <c r="N17" s="6"/>
       <c r="O17" s="6"/>
@@ -2918,7 +3035,7 @@
       <c r="K18" s="4"/>
       <c r="L18" s="4"/>
       <c r="M18" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N18" s="4">
         <v>4</v>
@@ -2927,7 +3044,7 @@
         <v>4</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
@@ -2950,7 +3067,7 @@
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
       <c r="M19" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N19" s="4">
         <v>4</v>
@@ -2959,7 +3076,7 @@
         <v>0</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
@@ -2981,10 +3098,12 @@
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4"/>
-      <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
-      <c r="O20" s="4"/>
-      <c r="P20" s="4"/>
+      <c r="M20" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="N20" s="6"/>
+      <c r="O20" s="6"/>
+      <c r="P20" s="6"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
@@ -3005,10 +3124,18 @@
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="4"/>
-      <c r="P21" s="4"/>
+      <c r="M21" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="N21" s="4">
+        <v>0</v>
+      </c>
+      <c r="O21" s="4">
+        <v>12</v>
+      </c>
+      <c r="P21" s="4" t="s">
+        <v>56</v>
+      </c>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
@@ -3071,7 +3198,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:W10"/>
+  <dimension ref="A1:W12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="4"/>
@@ -3141,15 +3268,6 @@
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
-      <c r="T1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="W1" s="1"/>
     </row>
     <row r="2" spans="1:23">
@@ -3183,13 +3301,22 @@
       <c r="J2" s="4">
         <v>7</v>
       </c>
+      <c r="T2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="3" spans="1:23">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" s="4">
         <v>3</v>
@@ -3215,14 +3342,14 @@
       <c r="J3" s="4">
         <v>5</v>
       </c>
-      <c r="M3" s="6" t="s">
-        <v>49</v>
+      <c r="M3" s="11" t="s">
+        <v>48</v>
       </c>
       <c r="N3" s="6"/>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="T3" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="U3" s="4">
         <v>12</v>
@@ -3236,13 +3363,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C4" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="4">
         <v>1</v>
@@ -3251,19 +3378,19 @@
         <v>1</v>
       </c>
       <c r="G4" s="4">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H4" s="4">
         <v>6</v>
       </c>
       <c r="I4" s="4">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="J4" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N4" s="4">
         <v>2</v>
@@ -3275,13 +3402,13 @@
         <v>17</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="U4" s="4">
         <v>7</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:23">
@@ -3289,10 +3416,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C5" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="4">
         <v>0</v>
@@ -3301,22 +3428,22 @@
         <v>0</v>
       </c>
       <c r="F5" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="4">
         <v>0</v>
       </c>
       <c r="H5" s="4">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I5" s="4">
-        <v>-14</v>
+        <v>-18</v>
       </c>
       <c r="J5" s="4">
         <v>0</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N5" s="4">
         <v>5</v>
@@ -3325,21 +3452,21 @@
         <v>0</v>
       </c>
       <c r="P5" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="T5" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="T5" s="4" t="s">
-        <v>71</v>
-      </c>
       <c r="U5" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:23">
-      <c r="M6" s="6" t="s">
-        <v>51</v>
+      <c r="M6" s="11" t="s">
+        <v>50</v>
       </c>
       <c r="N6" s="6"/>
       <c r="O6" s="6"/>
@@ -3356,12 +3483,12 @@
         <v>0</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:23">
       <c r="M8" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N8" s="4">
         <v>1</v>
@@ -3370,12 +3497,12 @@
         <v>1</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:23">
-      <c r="M9" s="6" t="s">
-        <v>72</v>
+      <c r="M9" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="N9" s="6"/>
       <c r="O9" s="6"/>
@@ -3392,7 +3519,29 @@
         <v>2</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23">
+      <c r="M11" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+    </row>
+    <row r="12" spans="1:23">
+      <c r="M12" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="N12" s="4">
+        <v>4</v>
+      </c>
+      <c r="O12" s="4">
+        <v>0</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -3443,7 +3592,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C2" s="4">
         <v>6</v>
@@ -3467,7 +3616,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C3" s="4">
         <v>5</v>
@@ -3482,7 +3631,7 @@
         <v>12</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
@@ -3493,7 +3642,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C4" s="4">
         <v>5</v>
@@ -3508,16 +3657,16 @@
         <v>11</v>
       </c>
       <c r="I4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
+        <v>3</v>
+      </c>
+      <c r="L4" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="J4" s="4">
-        <v>0</v>
-      </c>
-      <c r="K4" s="4">
-        <v>3</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>76</v>
       </c>
       <c r="M4" s="4"/>
     </row>
@@ -3526,7 +3675,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C5" s="4">
         <v>5</v>
@@ -3541,7 +3690,7 @@
         <v>9</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J5" s="4">
         <v>2</v>
@@ -3550,7 +3699,7 @@
         <v>1</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3558,7 +3707,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C6" s="4">
         <v>3</v>
@@ -3573,7 +3722,7 @@
         <v>7</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J6" s="4">
         <v>0</v>
@@ -3582,7 +3731,7 @@
         <v>3</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3590,7 +3739,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C7" s="4">
         <v>5</v>
@@ -3605,7 +3754,7 @@
         <v>3</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J7" s="4">
         <v>3</v>
@@ -3614,7 +3763,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -3622,7 +3771,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C8" s="4">
         <v>4</v>
@@ -3637,7 +3786,7 @@
         <v>3</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
@@ -3648,7 +3797,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C9" s="4">
         <v>5</v>
@@ -3663,7 +3812,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J9" s="4">
         <v>2</v>
@@ -3672,7 +3821,7 @@
         <v>1</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3680,7 +3829,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C10" s="4">
         <v>4</v>
@@ -3695,7 +3844,7 @@
         <v>0</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J10" s="4">
         <v>1</v>
@@ -3704,7 +3853,7 @@
         <v>2</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3715,7 +3864,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="I11" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J11" s="4">
         <v>0</v>
@@ -3724,7 +3873,7 @@
         <v>3</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -3735,7 +3884,7 @@
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="I12" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
@@ -3749,7 +3898,7 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="I13" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J13" s="4">
         <v>2</v>
@@ -3758,13 +3907,13 @@
         <v>1</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="4"/>
       <c r="I14" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J14" s="4">
         <v>1</v>
@@ -3773,28 +3922,28 @@
         <v>2</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="4"/>
       <c r="I15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="J15" s="4">
+        <v>3</v>
+      </c>
+      <c r="K15" s="4">
+        <v>0</v>
+      </c>
+      <c r="L15" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="J15" s="4">
-        <v>3</v>
-      </c>
-      <c r="K15" s="4">
-        <v>0</v>
-      </c>
-      <c r="L15" s="4" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J16" s="4">
         <v>3</v>
@@ -3803,13 +3952,13 @@
         <v>0</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="4"/>
       <c r="I17" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
@@ -3818,7 +3967,7 @@
     <row r="18" spans="1:12">
       <c r="A18" s="4"/>
       <c r="I18" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J18" s="4">
         <v>0</v>
@@ -3827,13 +3976,13 @@
         <v>3</v>
       </c>
       <c r="L18" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="4"/>
       <c r="I19" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J19" s="4">
         <v>0</v>
@@ -3842,13 +3991,13 @@
         <v>3</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="4"/>
       <c r="I20" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J20" s="4">
         <v>3</v>
@@ -3857,13 +4006,13 @@
         <v>0</v>
       </c>
       <c r="L20" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="4"/>
       <c r="I21" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
@@ -3872,7 +4021,7 @@
     <row r="22" spans="1:12">
       <c r="A22" s="4"/>
       <c r="I22" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J22" s="4">
         <v>3</v>
@@ -3881,12 +4030,12 @@
         <v>0</v>
       </c>
       <c r="L22" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="I23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J23" s="4">
         <v>3</v>
@@ -3895,26 +4044,26 @@
         <v>0</v>
       </c>
       <c r="L23" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:12">
       <c r="I24" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J24" s="4">
+        <v>3</v>
+      </c>
+      <c r="K24" s="4">
+        <v>0</v>
+      </c>
+      <c r="L24" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="J24" s="4">
-        <v>3</v>
-      </c>
-      <c r="K24" s="4">
-        <v>0</v>
-      </c>
-      <c r="L24" s="4" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="25" spans="1:12">
       <c r="I25" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
@@ -3922,7 +4071,7 @@
     </row>
     <row r="26" spans="1:12">
       <c r="I26" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J26" s="4">
         <v>3</v>
@@ -3931,12 +4080,12 @@
         <v>0</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:12">
       <c r="I27" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J27" s="4">
         <v>1</v>
@@ -3945,12 +4094,12 @@
         <v>2</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:12">
       <c r="I28" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J28" s="4">
         <v>0</v>
@@ -3959,12 +4108,12 @@
         <v>3</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:12">
       <c r="I29" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J29" s="4">
         <v>0</v>
@@ -3973,7 +4122,7 @@
         <v>3</v>
       </c>
       <c r="L29" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización de cronograma y datos de junio
</commit_message>
<xml_diff>
--- a/CAMPEONATO CACMQ 2026 (1).xlsx
+++ b/CAMPEONATO CACMQ 2026 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\CACMQ\JORNADAS DEPORTIVAS 2026 MAYO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADCAEB5-4165-4E6E-A37E-B77366EB379E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B8B0DB4-25C4-42D7-BB95-ABB6FF45A2E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="110">
   <si>
     <t>N</t>
   </si>
@@ -93,9 +93,6 @@
     <t>GAT-S</t>
   </si>
   <si>
-    <t>15 DE MAYO</t>
-  </si>
-  <si>
     <t>LUIS BARAJA</t>
   </si>
   <si>
@@ -141,9 +138,6 @@
     <t>26 DE MAYO</t>
   </si>
   <si>
-    <t>29DE MAYO</t>
-  </si>
-  <si>
     <t>01 DE JUNIO</t>
   </si>
   <si>
@@ -276,24 +270,15 @@
     <t>SOLO PANAS</t>
   </si>
   <si>
-    <t>22 DE MAYO</t>
-  </si>
-  <si>
     <t>BATE Y SALE</t>
   </si>
   <si>
-    <t>29 DE MAYO</t>
-  </si>
-  <si>
     <t>04 DE JUNIO</t>
   </si>
   <si>
     <t xml:space="preserve">ADMINISTRATIVOS </t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>05 DE JUNIO</t>
   </si>
   <si>
@@ -316,13 +301,79 @@
   </si>
   <si>
     <t>8 DE JUNIO  /DIFERIDO/</t>
+  </si>
+  <si>
+    <t>09 DE JUNIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          27 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">          28 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          26 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         20 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         19 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        18 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        28 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        20 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">               19 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                 22 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                  27 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                   29 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">            29 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">               26 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">              21 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">              18 DE MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">            15 DE MAYO</t>
+  </si>
+  <si>
+    <t>10 DE JUNIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      10 DE JUNIO</t>
+  </si>
+  <si>
+    <t>11 DE JUNIO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -355,6 +406,20 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -416,7 +481,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -444,19 +509,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1">
@@ -465,7 +518,25 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -963,7 +1034,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W35"/>
+  <dimension ref="A1:T40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="4" customWidth="1"/>
@@ -978,13 +1049,13 @@
     <col min="13" max="13" width="33" style="4" customWidth="1"/>
     <col min="14" max="15" width="6" style="4" customWidth="1"/>
     <col min="16" max="16" width="33" style="4" customWidth="1"/>
-    <col min="17" max="20" width="9.109375" style="4"/>
-    <col min="21" max="21" width="28.21875" style="4" customWidth="1"/>
-    <col min="22" max="22" width="9.109375" style="4"/>
-    <col min="23" max="23" width="18.5546875" style="4" customWidth="1"/>
+    <col min="17" max="17" width="9.109375" style="4"/>
+    <col min="18" max="18" width="28.21875" style="4" customWidth="1"/>
+    <col min="19" max="19" width="9.109375" style="4"/>
+    <col min="20" max="20" width="18.5546875" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="7" customFormat="1">
+    <row r="1" spans="1:20" s="7" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1024,284 +1095,281 @@
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-    </row>
-    <row r="2" spans="1:23">
+    </row>
+    <row r="2" spans="1:20" ht="15.6">
       <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="12">
         <v>6</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="12">
         <v>6</v>
       </c>
-      <c r="E2" s="4">
-        <v>0</v>
-      </c>
-      <c r="F2" s="4">
-        <v>0</v>
-      </c>
-      <c r="G2" s="4">
+      <c r="E2" s="12">
+        <v>0</v>
+      </c>
+      <c r="F2" s="12">
+        <v>0</v>
+      </c>
+      <c r="G2" s="12">
         <v>27</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="12">
         <v>9</v>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="12">
         <v>18</v>
       </c>
-      <c r="J2" s="4">
+      <c r="J2" s="12">
         <v>18</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="W2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:23">
+    <row r="3" spans="1:20" ht="15.6">
       <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="12">
         <v>6</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="12">
         <v>5</v>
       </c>
-      <c r="E3" s="4">
-        <v>0</v>
-      </c>
-      <c r="F3" s="4">
-        <v>1</v>
-      </c>
-      <c r="G3" s="4">
+      <c r="E3" s="12">
+        <v>0</v>
+      </c>
+      <c r="F3" s="12">
+        <v>1</v>
+      </c>
+      <c r="G3" s="12">
         <v>27</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="12">
         <v>7</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="12">
         <v>20</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="12">
         <v>15</v>
       </c>
-      <c r="M3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="N3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="9" t="s">
+        <v>106</v>
+      </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
-      <c r="U3" s="4" t="s">
+      <c r="R3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="V3" s="4">
+      <c r="S3" s="4">
         <v>11</v>
       </c>
-      <c r="W3" s="4" t="s">
+      <c r="T3" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:23">
+    <row r="4" spans="1:20" ht="15.6">
       <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="12">
         <v>5</v>
       </c>
-      <c r="D4" s="4">
-        <v>4</v>
-      </c>
-      <c r="E4" s="4">
-        <v>1</v>
-      </c>
-      <c r="F4" s="4">
-        <v>0</v>
-      </c>
-      <c r="G4" s="4">
+      <c r="D4" s="12">
+        <v>4</v>
+      </c>
+      <c r="E4" s="12">
+        <v>1</v>
+      </c>
+      <c r="F4" s="12">
+        <v>0</v>
+      </c>
+      <c r="G4" s="12">
         <v>17</v>
       </c>
-      <c r="H4" s="4">
-        <v>2</v>
-      </c>
-      <c r="I4" s="4">
+      <c r="H4" s="12">
+        <v>2</v>
+      </c>
+      <c r="I4" s="12">
         <v>15</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="12">
         <v>13</v>
       </c>
       <c r="M4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" s="4">
+        <v>3</v>
+      </c>
+      <c r="O4" s="4">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="N4" s="4">
-        <v>3</v>
-      </c>
-      <c r="O4" s="4">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="U4" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="V4" s="4">
+      <c r="R4" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="S4" s="4">
         <v>9</v>
       </c>
-      <c r="W4" s="4" t="s">
+      <c r="T4" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:23">
+    <row r="5" spans="1:20" ht="15.6">
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="4">
+      <c r="B5" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="12">
         <v>5</v>
       </c>
-      <c r="D5" s="4">
-        <v>2</v>
-      </c>
-      <c r="E5" s="4">
-        <v>1</v>
-      </c>
-      <c r="F5" s="4">
-        <v>2</v>
-      </c>
-      <c r="G5" s="4">
+      <c r="D5" s="12">
+        <v>2</v>
+      </c>
+      <c r="E5" s="12">
+        <v>1</v>
+      </c>
+      <c r="F5" s="12">
+        <v>2</v>
+      </c>
+      <c r="G5" s="12">
         <v>13</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="12">
         <v>8</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="12">
         <v>5</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="12">
         <v>7</v>
       </c>
-      <c r="M5" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="N5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="9" t="s">
+        <v>105</v>
+      </c>
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
-      <c r="U5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="V5" s="4">
+      <c r="R5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="S5" s="4">
         <v>6</v>
       </c>
-      <c r="W5" s="4" t="s">
+      <c r="T5" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:23">
+    <row r="6" spans="1:20" ht="15.6">
       <c r="A6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="4">
+      <c r="B6" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="12">
         <v>5</v>
       </c>
-      <c r="D6" s="4">
-        <v>2</v>
-      </c>
-      <c r="E6" s="4">
-        <v>1</v>
-      </c>
-      <c r="F6" s="4">
-        <v>2</v>
-      </c>
-      <c r="G6" s="4">
+      <c r="D6" s="12">
+        <v>2</v>
+      </c>
+      <c r="E6" s="12">
+        <v>1</v>
+      </c>
+      <c r="F6" s="12">
+        <v>2</v>
+      </c>
+      <c r="G6" s="12">
         <v>5</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="12">
         <v>12</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="12">
         <v>-7</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="12">
         <v>7</v>
       </c>
       <c r="M6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="N6" s="4">
+        <v>3</v>
+      </c>
+      <c r="O6" s="4">
+        <v>1</v>
+      </c>
+      <c r="P6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="N6" s="4">
-        <v>3</v>
-      </c>
-      <c r="O6" s="4">
-        <v>1</v>
-      </c>
-      <c r="P6" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="U6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="V6" s="4">
-        <v>4</v>
-      </c>
-      <c r="W6" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23">
+      <c r="R6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="S6" s="4">
+        <v>4</v>
+      </c>
+      <c r="T6" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="15.6">
       <c r="A7" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="4">
+      <c r="B7" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="12">
         <v>6</v>
       </c>
-      <c r="D7" s="4">
-        <v>1</v>
-      </c>
-      <c r="E7" s="4">
-        <v>1</v>
-      </c>
-      <c r="F7" s="4">
-        <v>4</v>
-      </c>
-      <c r="G7" s="4">
+      <c r="D7" s="12">
+        <v>1</v>
+      </c>
+      <c r="E7" s="12">
+        <v>1</v>
+      </c>
+      <c r="F7" s="12">
+        <v>4</v>
+      </c>
+      <c r="G7" s="12">
         <v>7</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="12">
         <v>14</v>
       </c>
-      <c r="I7" s="4">
+      <c r="I7" s="12">
         <v>-7</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="12">
         <v>4</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N7" s="4">
         <v>4</v>
@@ -1310,42 +1378,42 @@
         <v>1</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" ht="15.6">
       <c r="A8" s="4">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="4">
+      <c r="B8" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="12">
         <v>5</v>
       </c>
-      <c r="D8" s="4">
-        <v>1</v>
-      </c>
-      <c r="E8" s="4">
-        <v>1</v>
-      </c>
-      <c r="F8" s="4">
-        <v>3</v>
-      </c>
-      <c r="G8" s="4">
+      <c r="D8" s="12">
+        <v>1</v>
+      </c>
+      <c r="E8" s="12">
+        <v>1</v>
+      </c>
+      <c r="F8" s="12">
+        <v>3</v>
+      </c>
+      <c r="G8" s="12">
         <v>8</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="12">
         <v>15</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="12">
         <v>-8</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="12">
         <v>4</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N8" s="4">
         <v>7</v>
@@ -1354,38 +1422,38 @@
         <v>0</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" ht="15.6">
       <c r="A9" s="4">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="4">
+      <c r="B9" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="12">
         <v>6</v>
       </c>
-      <c r="D9" s="4">
-        <v>1</v>
-      </c>
-      <c r="E9" s="4">
-        <v>1</v>
-      </c>
-      <c r="F9" s="4">
-        <v>4</v>
-      </c>
-      <c r="G9" s="4">
+      <c r="D9" s="12">
+        <v>1</v>
+      </c>
+      <c r="E9" s="12">
+        <v>1</v>
+      </c>
+      <c r="F9" s="12">
+        <v>4</v>
+      </c>
+      <c r="G9" s="12">
         <v>7</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="12">
         <v>18</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="12">
         <v>-11</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="12">
         <v>4</v>
       </c>
       <c r="M9" s="4" t="s">
@@ -1398,48 +1466,48 @@
         <v>0</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" ht="15.6">
       <c r="A10" s="4">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="4">
+      <c r="B10" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="12">
         <v>5</v>
       </c>
-      <c r="D10" s="4">
-        <v>0</v>
-      </c>
-      <c r="E10" s="4">
-        <v>0</v>
-      </c>
-      <c r="F10" s="4">
+      <c r="D10" s="12">
+        <v>0</v>
+      </c>
+      <c r="E10" s="12">
+        <v>0</v>
+      </c>
+      <c r="F10" s="12">
         <v>5</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="12">
         <v>7</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="12">
         <v>27</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="12">
         <v>-20</v>
       </c>
-      <c r="J10" s="4">
-        <v>0</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="N10" s="6"/>
+      <c r="J10" s="12">
+        <v>0</v>
+      </c>
+      <c r="M10" s="6"/>
+      <c r="N10" s="9" t="s">
+        <v>104</v>
+      </c>
       <c r="O10" s="6"/>
       <c r="P10" s="6"/>
     </row>
-    <row r="11" spans="1:23">
+    <row r="11" spans="1:20">
       <c r="M11" s="4" t="s">
         <v>16</v>
       </c>
@@ -1450,12 +1518,12 @@
         <v>2</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20">
       <c r="M12" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N12" s="4">
         <v>1</v>
@@ -1467,7 +1535,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:23">
+    <row r="13" spans="1:20">
       <c r="M13" s="4" t="s">
         <v>14</v>
       </c>
@@ -1478,20 +1546,20 @@
         <v>0</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23">
-      <c r="M14" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N14" s="6"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20">
+      <c r="M14" s="6"/>
+      <c r="N14" s="9" t="s">
+        <v>103</v>
+      </c>
       <c r="O14" s="6"/>
       <c r="P14" s="6"/>
     </row>
-    <row r="15" spans="1:23">
+    <row r="15" spans="1:20">
       <c r="M15" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N15" s="4">
         <v>4</v>
@@ -1500,12 +1568,12 @@
         <v>3</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20">
       <c r="M16" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N16" s="4">
         <v>3</v>
@@ -1514,10 +1582,10 @@
         <v>4</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="13:17">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="13:16">
       <c r="M17" s="4" t="s">
         <v>14</v>
       </c>
@@ -1528,10 +1596,10 @@
         <v>0</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="13:17">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="13:16">
       <c r="M18" s="4" t="s">
         <v>16</v>
       </c>
@@ -1545,17 +1613,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="13:17">
-      <c r="M19" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="N19" s="6"/>
+    <row r="19" spans="13:16">
+      <c r="M19" s="5"/>
+      <c r="N19" s="9" t="s">
+        <v>102</v>
+      </c>
       <c r="O19" s="6"/>
       <c r="P19" s="6"/>
     </row>
-    <row r="20" spans="13:17">
+    <row r="20" spans="13:16">
       <c r="M20" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N20" s="4">
         <v>1</v>
@@ -1564,10 +1632,10 @@
         <v>1</v>
       </c>
       <c r="P20" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="13:17">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="13:16">
       <c r="M21" s="4" t="s">
         <v>16</v>
       </c>
@@ -1578,10 +1646,10 @@
         <v>0</v>
       </c>
       <c r="P21" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="22" spans="13:17">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="13:16">
       <c r="M22" s="4" t="s">
         <v>14</v>
       </c>
@@ -1592,20 +1660,20 @@
         <v>2</v>
       </c>
       <c r="P22" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="13:17">
-      <c r="M23" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="N23" s="6"/>
-      <c r="O23" s="6"/>
-      <c r="P23" s="6"/>
-    </row>
-    <row r="24" spans="13:17">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="13:16">
+      <c r="M23" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="N23" s="17"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="17"/>
+    </row>
+    <row r="24" spans="13:16">
       <c r="M24" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N24" s="4">
         <v>6</v>
@@ -1614,12 +1682,12 @@
         <v>2</v>
       </c>
       <c r="P24" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" spans="13:17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="13:16">
       <c r="M25" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N25" s="4">
         <v>0</v>
@@ -1631,9 +1699,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="13:17">
+    <row r="26" spans="13:16">
       <c r="M26" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N26" s="4">
         <v>0</v>
@@ -1642,10 +1710,10 @@
         <v>1</v>
       </c>
       <c r="P26" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="27" spans="13:17">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="13:16">
       <c r="M27" s="4" t="s">
         <v>16</v>
       </c>
@@ -1656,34 +1724,34 @@
         <v>1</v>
       </c>
       <c r="P27" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="13:16">
+      <c r="M28" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="N28" s="17"/>
+      <c r="O28" s="17"/>
+      <c r="P28" s="17"/>
+    </row>
+    <row r="29" spans="13:16">
+      <c r="M29" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="N29" s="8">
+        <v>1</v>
+      </c>
+      <c r="O29" s="8">
+        <v>0</v>
+      </c>
+      <c r="P29" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="13:17">
-      <c r="M28" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="N28" s="6"/>
-      <c r="O28" s="6"/>
-      <c r="P28" s="6"/>
-    </row>
-    <row r="29" spans="13:17">
-      <c r="M29" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="N29" s="8">
-        <v>1</v>
-      </c>
-      <c r="O29" s="8">
-        <v>0</v>
-      </c>
-      <c r="P29" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" spans="13:17">
+    <row r="30" spans="13:16">
       <c r="M30" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N30" s="4">
         <v>2</v>
@@ -1694,13 +1762,10 @@
       <c r="P30" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="Q30" s="8" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="31" spans="13:17">
+    </row>
+    <row r="31" spans="13:16">
       <c r="M31" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N31" s="4">
         <v>1</v>
@@ -1709,18 +1774,19 @@
         <v>1</v>
       </c>
       <c r="P31" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="32" spans="13:17">
-      <c r="M32" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="N32" s="6"/>
-      <c r="O32" s="6"/>
-      <c r="P32" s="6"/>
-    </row>
-    <row r="33" spans="13:16">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="13:16">
+      <c r="M32" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="N32" s="17"/>
+      <c r="O32" s="17"/>
+      <c r="P32" s="17"/>
+    </row>
+    <row r="33" spans="1:16">
+      <c r="A33" s="15"/>
       <c r="M33" s="4" t="s">
         <v>16</v>
       </c>
@@ -1731,26 +1797,26 @@
         <v>1</v>
       </c>
       <c r="P33" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="34" spans="13:16">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16">
       <c r="M34" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N34" s="4">
+        <v>3</v>
+      </c>
+      <c r="O34" s="4">
+        <v>1</v>
+      </c>
+      <c r="P34" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16">
+      <c r="M35" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="N34" s="4">
-        <v>3</v>
-      </c>
-      <c r="O34" s="4">
-        <v>1</v>
-      </c>
-      <c r="P34" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="35" spans="13:16">
-      <c r="M35" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="N35" s="4">
         <v>6</v>
@@ -1759,17 +1825,65 @@
         <v>2</v>
       </c>
       <c r="P35" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16">
+      <c r="M36" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="N36" s="17"/>
+      <c r="O36" s="17"/>
+      <c r="P36" s="17"/>
+    </row>
+    <row r="37" spans="1:16">
+      <c r="M37" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N37" s="8"/>
+      <c r="O37" s="8"/>
+      <c r="P37" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16">
+      <c r="M38" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="P38" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16">
+      <c r="M39" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="P39" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16">
+      <c r="M40" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="P40" s="4" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="M23:P23"/>
+    <mergeCell ref="M28:P28"/>
+    <mergeCell ref="M32:P32"/>
+    <mergeCell ref="M36:P36"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:V27"/>
+  <dimension ref="A1:V32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="27.88671875" style="4" customWidth="1"/>
@@ -1778,7 +1892,7 @@
     <col min="5" max="5" width="3.88671875" customWidth="1"/>
     <col min="6" max="7" width="4.21875" customWidth="1"/>
     <col min="8" max="8" width="4.33203125" customWidth="1"/>
-    <col min="9" max="9" width="3.77734375" customWidth="1"/>
+    <col min="9" max="9" width="6.6640625" customWidth="1"/>
     <col min="10" max="10" width="3.88671875" customWidth="1"/>
     <col min="13" max="13" width="27.88671875" style="4" customWidth="1"/>
     <col min="14" max="14" width="5.33203125" style="4" customWidth="1"/>
@@ -1790,7 +1904,7 @@
     <col min="22" max="22" width="18.33203125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="14" customFormat="1">
+    <row r="1" spans="1:22" s="10" customFormat="1" ht="18">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -1821,557 +1935,599 @@
       <c r="J1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="15" t="s">
+      <c r="M1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="N1" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="O1" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="P1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+    </row>
+    <row r="2" spans="1:22" ht="18">
+      <c r="A2" s="14">
+        <v>1</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="14">
+        <v>5</v>
+      </c>
+      <c r="D2" s="14">
+        <v>3</v>
+      </c>
+      <c r="E2" s="14">
+        <v>1</v>
+      </c>
+      <c r="F2" s="14">
+        <v>1</v>
+      </c>
+      <c r="G2" s="14">
+        <v>20</v>
+      </c>
+      <c r="H2" s="14">
+        <v>16</v>
+      </c>
+      <c r="I2" s="14">
+        <v>4</v>
+      </c>
+      <c r="J2" s="14">
+        <v>10</v>
+      </c>
+      <c r="T2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="U2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="V2" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" ht="18">
+      <c r="A3" s="14">
+        <v>2</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="O1" s="15" t="s">
+      <c r="C3" s="14">
+        <v>3</v>
+      </c>
+      <c r="D3" s="14">
+        <v>3</v>
+      </c>
+      <c r="E3" s="14">
+        <v>0</v>
+      </c>
+      <c r="F3" s="14">
+        <v>0</v>
+      </c>
+      <c r="G3" s="14">
+        <v>15</v>
+      </c>
+      <c r="H3" s="14">
+        <v>2</v>
+      </c>
+      <c r="I3" s="14">
+        <v>13</v>
+      </c>
+      <c r="J3" s="14">
+        <v>9</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="T3" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="P1" s="15"/>
-      <c r="T1" s="15"/>
-      <c r="U1" s="15"/>
-      <c r="V1" s="15"/>
-    </row>
-    <row r="2" spans="1:22">
-      <c r="A2" s="9">
-        <v>1</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="9">
-        <v>5</v>
-      </c>
-      <c r="D2" s="9">
-        <v>3</v>
-      </c>
-      <c r="E2" s="9">
-        <v>1</v>
-      </c>
-      <c r="F2" s="9">
-        <v>1</v>
-      </c>
-      <c r="G2" s="9">
-        <v>20</v>
-      </c>
-      <c r="H2" s="9">
-        <v>16</v>
-      </c>
-      <c r="I2" s="9">
-        <v>4</v>
-      </c>
-      <c r="J2" s="9">
-        <v>10</v>
-      </c>
-      <c r="T2" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="U2" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="V2" s="15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="A3" s="9">
-        <v>2</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="9">
-        <v>3</v>
-      </c>
-      <c r="D3" s="9">
-        <v>3</v>
-      </c>
-      <c r="E3" s="9">
-        <v>0</v>
-      </c>
-      <c r="F3" s="9">
-        <v>0</v>
-      </c>
-      <c r="G3" s="9">
-        <v>15</v>
-      </c>
-      <c r="H3" s="9">
-        <v>2</v>
-      </c>
-      <c r="I3" s="9">
-        <v>13</v>
-      </c>
-      <c r="J3" s="9">
-        <v>9</v>
-      </c>
-      <c r="M3" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-      <c r="T3" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="U3" s="4">
         <v>11</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22">
-      <c r="A4" s="9">
-        <v>3</v>
-      </c>
-      <c r="B4" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" ht="18">
+      <c r="A4" s="14">
+        <v>3</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="14">
+        <v>3</v>
+      </c>
+      <c r="D4" s="14">
+        <v>2</v>
+      </c>
+      <c r="E4" s="14">
+        <v>1</v>
+      </c>
+      <c r="F4" s="14">
+        <v>0</v>
+      </c>
+      <c r="G4" s="14">
+        <v>11</v>
+      </c>
+      <c r="H4" s="14">
+        <v>9</v>
+      </c>
+      <c r="I4" s="14">
+        <v>8</v>
+      </c>
+      <c r="J4" s="14">
+        <v>7</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="N4" s="4">
+        <v>4</v>
+      </c>
+      <c r="O4" s="4">
+        <v>4</v>
+      </c>
+      <c r="P4" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="9">
-        <v>3</v>
-      </c>
-      <c r="D4" s="9">
-        <v>2</v>
-      </c>
-      <c r="E4" s="9">
-        <v>1</v>
-      </c>
-      <c r="F4" s="9">
-        <v>0</v>
-      </c>
-      <c r="G4" s="9">
-        <v>11</v>
-      </c>
-      <c r="H4" s="9">
-        <v>9</v>
-      </c>
-      <c r="I4" s="9">
-        <v>8</v>
-      </c>
-      <c r="J4" s="9">
-        <v>7</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="N4" s="9">
-        <v>4</v>
-      </c>
-      <c r="O4" s="9">
-        <v>4</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>45</v>
-      </c>
       <c r="T4" s="4" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="U4" s="4">
         <v>7</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22">
-      <c r="A5" s="9">
-        <v>4</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="9">
-        <v>4</v>
-      </c>
-      <c r="D5" s="9">
-        <v>2</v>
-      </c>
-      <c r="E5" s="9">
-        <v>1</v>
-      </c>
-      <c r="F5" s="9">
-        <v>1</v>
-      </c>
-      <c r="G5" s="9">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="18">
+      <c r="A5" s="14">
+        <v>4</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="14">
+        <v>4</v>
+      </c>
+      <c r="D5" s="14">
+        <v>2</v>
+      </c>
+      <c r="E5" s="14">
+        <v>1</v>
+      </c>
+      <c r="F5" s="14">
+        <v>1</v>
+      </c>
+      <c r="G5" s="14">
         <v>12</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="14">
         <v>7</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="14">
         <v>5</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="14">
         <v>7</v>
       </c>
-      <c r="M5" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
+      <c r="M5" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="N5" s="18"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
       <c r="T5" s="4" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="U5" s="4">
         <v>7</v>
       </c>
       <c r="V5" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="18">
+      <c r="A6" s="14">
+        <v>5</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="6" spans="1:22">
-      <c r="A6" s="9">
-        <v>5</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="9">
-        <v>4</v>
-      </c>
-      <c r="D6" s="9">
-        <v>0</v>
-      </c>
-      <c r="E6" s="9">
-        <v>2</v>
-      </c>
-      <c r="F6" s="9">
-        <v>2</v>
-      </c>
-      <c r="G6" s="9">
+      <c r="C6" s="14">
+        <v>4</v>
+      </c>
+      <c r="D6" s="14">
+        <v>0</v>
+      </c>
+      <c r="E6" s="14">
+        <v>2</v>
+      </c>
+      <c r="F6" s="14">
+        <v>2</v>
+      </c>
+      <c r="G6" s="14">
         <v>8</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="14">
         <v>14</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="14">
         <v>-6</v>
       </c>
-      <c r="J6" s="9">
-        <v>2</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="N6" s="9">
-        <v>3</v>
-      </c>
-      <c r="O6" s="9">
+      <c r="J6" s="14">
+        <v>2</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="N6" s="4">
+        <v>3</v>
+      </c>
+      <c r="O6" s="4">
         <v>6</v>
       </c>
-      <c r="P6" s="9" t="s">
-        <v>43</v>
+      <c r="P6" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="U6" s="4">
         <v>6</v>
       </c>
       <c r="V6" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="18">
+      <c r="A7" s="14">
+        <v>6</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="14">
+        <v>4</v>
+      </c>
+      <c r="D7" s="14">
+        <v>0</v>
+      </c>
+      <c r="E7" s="14">
+        <v>1</v>
+      </c>
+      <c r="F7" s="14">
+        <v>3</v>
+      </c>
+      <c r="G7" s="14">
+        <v>7</v>
+      </c>
+      <c r="H7" s="14">
+        <v>17</v>
+      </c>
+      <c r="I7" s="14">
+        <v>-10</v>
+      </c>
+      <c r="J7" s="14">
+        <v>1</v>
+      </c>
+      <c r="M7" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+    </row>
+    <row r="8" spans="1:22" ht="18">
+      <c r="A8" s="14">
+        <v>7</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="14">
+        <v>3</v>
+      </c>
+      <c r="D8" s="14">
+        <v>0</v>
+      </c>
+      <c r="E8" s="14">
+        <v>0</v>
+      </c>
+      <c r="F8" s="14">
+        <v>3</v>
+      </c>
+      <c r="G8" s="14">
+        <v>4</v>
+      </c>
+      <c r="H8" s="14">
+        <v>19</v>
+      </c>
+      <c r="I8" s="14">
+        <v>-15</v>
+      </c>
+      <c r="J8" s="14">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="N8" s="4">
+        <v>3</v>
+      </c>
+      <c r="O8" s="4">
+        <v>2</v>
+      </c>
+      <c r="P8" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22">
+      <c r="M9" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
+    </row>
+    <row r="10" spans="1:22">
+      <c r="M10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N10" s="4">
+        <v>0</v>
+      </c>
+      <c r="O10" s="4">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:22">
-      <c r="A7" s="9">
+    <row r="11" spans="1:22">
+      <c r="M11" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="N11" s="18"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="18"/>
+    </row>
+    <row r="12" spans="1:22">
+      <c r="M12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N12" s="4">
+        <v>5</v>
+      </c>
+      <c r="O12" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="P12" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
+      <c r="M13" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="N13" s="18"/>
+      <c r="O13" s="18"/>
+      <c r="P13" s="18"/>
+    </row>
+    <row r="14" spans="1:22">
+      <c r="M14" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="9">
-        <v>4</v>
-      </c>
-      <c r="D7" s="9">
-        <v>0</v>
-      </c>
-      <c r="E7" s="9">
-        <v>1</v>
-      </c>
-      <c r="F7" s="9">
-        <v>3</v>
-      </c>
-      <c r="G7" s="9">
+      <c r="N14" s="4">
+        <v>0</v>
+      </c>
+      <c r="O14" s="4">
+        <v>9</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22">
+      <c r="M15" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="N15" s="18"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="18"/>
+    </row>
+    <row r="16" spans="1:22">
+      <c r="M16" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="N16" s="4">
+        <v>5</v>
+      </c>
+      <c r="O16" s="4">
+        <v>3</v>
+      </c>
+      <c r="P16" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="13:16">
+      <c r="M17" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="18"/>
+    </row>
+    <row r="18" spans="13:16">
+      <c r="M18" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="N18" s="4">
+        <v>5</v>
+      </c>
+      <c r="O18" s="4">
+        <v>1</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="13:16">
+      <c r="M19" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="N19" s="4">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4">
+        <v>3</v>
+      </c>
+      <c r="P19" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="13:16">
+      <c r="M20" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="N20" s="18"/>
+      <c r="O20" s="18"/>
+      <c r="P20" s="18"/>
+    </row>
+    <row r="21" spans="13:16">
+      <c r="M21" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="N21" s="4">
+        <v>0</v>
+      </c>
+      <c r="O21" s="4">
+        <v>3</v>
+      </c>
+      <c r="P21" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="13:16">
+      <c r="M22" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="N22" s="18"/>
+      <c r="O22" s="18"/>
+      <c r="P22" s="18"/>
+    </row>
+    <row r="23" spans="13:16">
+      <c r="M23" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="N23" s="4">
+        <v>1</v>
+      </c>
+      <c r="O23" s="4">
+        <v>4</v>
+      </c>
+      <c r="P23" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="13:16">
+      <c r="M24" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="N24" s="18"/>
+      <c r="O24" s="18"/>
+      <c r="P24" s="18"/>
+    </row>
+    <row r="25" spans="13:16">
+      <c r="M25" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="N25" s="4">
+        <v>3</v>
+      </c>
+      <c r="O25" s="4">
+        <v>3</v>
+      </c>
+      <c r="P25" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="13:16">
+      <c r="M26" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="N26" s="18"/>
+      <c r="O26" s="18"/>
+      <c r="P26" s="18"/>
+    </row>
+    <row r="27" spans="13:16">
+      <c r="M27" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="N27" s="4">
+        <v>3</v>
+      </c>
+      <c r="O27" s="4">
         <v>7</v>
       </c>
-      <c r="H7" s="9">
-        <v>17</v>
-      </c>
-      <c r="I7" s="9">
-        <v>-10</v>
-      </c>
-      <c r="J7" s="9">
-        <v>1</v>
-      </c>
-      <c r="M7" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
-    </row>
-    <row r="8" spans="1:22">
-      <c r="A8" s="9">
-        <v>7</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="9">
-        <v>3</v>
-      </c>
-      <c r="D8" s="9">
-        <v>0</v>
-      </c>
-      <c r="E8" s="9">
-        <v>0</v>
-      </c>
-      <c r="F8" s="9">
-        <v>3</v>
-      </c>
-      <c r="G8" s="9">
-        <v>4</v>
-      </c>
-      <c r="H8" s="9">
-        <v>19</v>
-      </c>
-      <c r="I8" s="9">
-        <v>-15</v>
-      </c>
-      <c r="J8" s="9">
-        <v>0</v>
-      </c>
-      <c r="M8" s="9" t="s">
+      <c r="P27" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="13:16">
+      <c r="M28" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="N28" s="18"/>
+      <c r="O28" s="18"/>
+      <c r="P28" s="18"/>
+    </row>
+    <row r="29" spans="13:16">
+      <c r="M29" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="P29" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="N8" s="9">
-        <v>3</v>
-      </c>
-      <c r="O8" s="9">
-        <v>2</v>
-      </c>
-      <c r="P8" s="9" t="s">
+    </row>
+    <row r="30" spans="13:16">
+      <c r="M30" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="P30" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:22">
-      <c r="M9" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="16"/>
-    </row>
-    <row r="10" spans="1:22">
-      <c r="M10" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="N10" s="9">
-        <v>0</v>
-      </c>
-      <c r="O10" s="9">
-        <v>0</v>
-      </c>
-      <c r="P10" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22">
-      <c r="M11" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="16"/>
-    </row>
-    <row r="12" spans="1:22">
-      <c r="M12" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="N12" s="9">
-        <v>5</v>
-      </c>
-      <c r="O12" s="9">
-        <v>6</v>
-      </c>
-      <c r="P12" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22">
-      <c r="M13" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="N13" s="16"/>
-      <c r="O13" s="16"/>
-      <c r="P13" s="16"/>
-    </row>
-    <row r="14" spans="1:22">
-      <c r="M14" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="N14" s="9">
-        <v>0</v>
-      </c>
-      <c r="O14" s="9">
-        <v>9</v>
-      </c>
-      <c r="P14" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22">
-      <c r="M15" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N15" s="16"/>
-      <c r="O15" s="16"/>
-      <c r="P15" s="16"/>
-    </row>
-    <row r="16" spans="1:22">
-      <c r="M16" s="9" t="s">
+    <row r="31" spans="13:16">
+      <c r="M31" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="N31" s="18"/>
+      <c r="O31" s="18"/>
+      <c r="P31" s="18"/>
+    </row>
+    <row r="32" spans="13:16">
+      <c r="M32" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="P32" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="N16" s="9">
-        <v>5</v>
-      </c>
-      <c r="O16" s="9">
-        <v>3</v>
-      </c>
-      <c r="P16" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="17" spans="13:16">
-      <c r="M17" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="N17" s="16"/>
-      <c r="O17" s="16"/>
-      <c r="P17" s="16"/>
-    </row>
-    <row r="18" spans="13:16">
-      <c r="M18" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="N18" s="9">
-        <v>5</v>
-      </c>
-      <c r="O18" s="9">
-        <v>1</v>
-      </c>
-      <c r="P18" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="13:16">
-      <c r="M19" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="N19" s="9">
-        <v>0</v>
-      </c>
-      <c r="O19" s="9">
-        <v>3</v>
-      </c>
-      <c r="P19" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="13:16">
-      <c r="M20" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N20" s="16"/>
-      <c r="O20" s="16"/>
-      <c r="P20" s="16"/>
-    </row>
-    <row r="21" spans="13:16">
-      <c r="M21" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="N21" s="9">
-        <v>0</v>
-      </c>
-      <c r="O21" s="9">
-        <v>3</v>
-      </c>
-      <c r="P21" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="22" spans="13:16">
-      <c r="M22" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="N22" s="16"/>
-      <c r="O22" s="16"/>
-      <c r="P22" s="16"/>
-    </row>
-    <row r="23" spans="13:16">
-      <c r="M23" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="N23" s="9">
-        <v>1</v>
-      </c>
-      <c r="O23" s="9">
-        <v>4</v>
-      </c>
-      <c r="P23" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="24" spans="13:16">
-      <c r="M24" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="N24" s="16"/>
-      <c r="O24" s="16"/>
-      <c r="P24" s="16"/>
-    </row>
-    <row r="25" spans="13:16">
-      <c r="M25" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="N25" s="9">
-        <v>3</v>
-      </c>
-      <c r="O25" s="9">
-        <v>3</v>
-      </c>
-      <c r="P25" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="26" spans="13:16">
-      <c r="M26" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="N26" s="16"/>
-      <c r="O26" s="16"/>
-      <c r="P26" s="16"/>
-    </row>
-    <row r="27" spans="13:16">
-      <c r="M27" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="N27" s="9">
-        <v>3</v>
-      </c>
-      <c r="O27" s="9">
-        <v>7</v>
-      </c>
-      <c r="P27" s="10" t="s">
-        <v>42</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
+    <mergeCell ref="M28:P28"/>
+    <mergeCell ref="M31:P31"/>
     <mergeCell ref="M13:P13"/>
     <mergeCell ref="M3:P3"/>
     <mergeCell ref="M5:P5"/>
@@ -2391,7 +2547,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="27.33203125" customWidth="1"/>
@@ -2454,7 +2610,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="S1" s="1"/>
     </row>
@@ -2463,7 +2619,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C2" s="4">
         <v>4</v>
@@ -2496,7 +2652,9 @@
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
+      <c r="R2" s="15" t="s">
+        <v>90</v>
+      </c>
       <c r="S2" s="4"/>
       <c r="T2" s="1" t="s">
         <v>11</v>
@@ -2513,7 +2671,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C3" s="4">
         <v>4</v>
@@ -2541,23 +2699,23 @@
       </c>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="N3" s="6"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="9" t="s">
+        <v>95</v>
+      </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="U3" s="4">
         <v>18</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -2565,7 +2723,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C4" s="4">
         <v>3</v>
@@ -2594,7 +2752,7 @@
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="N4" s="4">
         <v>2</v>
@@ -2603,19 +2761,19 @@
         <v>2</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="U4" s="4">
         <v>11</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -2623,7 +2781,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C5" s="4">
         <v>3</v>
@@ -2651,23 +2809,23 @@
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
-      <c r="M5" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="N5" s="6"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="9" t="s">
+        <v>94</v>
+      </c>
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="U5" s="4">
         <v>2</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:22">
@@ -2675,7 +2833,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C6" s="4">
         <v>3</v>
@@ -2704,7 +2862,7 @@
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="N6" s="4">
         <v>4</v>
@@ -2713,19 +2871,19 @@
         <v>2</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="U6" s="4">
         <v>2</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -2733,7 +2891,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C7" s="4">
         <v>3</v>
@@ -2761,10 +2919,10 @@
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
-      <c r="M7" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="N7" s="6"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="9" t="s">
+        <v>93</v>
+      </c>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
       <c r="Q7" s="4"/>
@@ -2788,7 +2946,7 @@
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="N8" s="4">
         <v>12</v>
@@ -2797,7 +2955,7 @@
         <v>1</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
@@ -2810,10 +2968,10 @@
       <c r="A9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
-      <c r="M9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="N9" s="6"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9" t="s">
+        <v>92</v>
+      </c>
       <c r="O9" s="6"/>
       <c r="P9" s="6"/>
       <c r="Q9" s="4"/>
@@ -2837,7 +2995,7 @@
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="N10" s="4">
         <v>10</v>
@@ -2846,11 +3004,11 @@
         <v>2</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="Q10" s="4"/>
       <c r="R10" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
@@ -2861,10 +3019,10 @@
       <c r="A11" s="4"/>
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
-      <c r="M11" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="N11" s="6"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9" t="s">
+        <v>89</v>
+      </c>
       <c r="O11" s="6"/>
       <c r="P11" s="6"/>
       <c r="Q11" s="4"/>
@@ -2879,7 +3037,7 @@
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N12" s="4">
         <v>3</v>
@@ -2888,7 +3046,7 @@
         <v>1</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
@@ -2901,10 +3059,10 @@
       <c r="A13" s="4"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="N13" s="6"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9" t="s">
+        <v>91</v>
+      </c>
       <c r="O13" s="6"/>
       <c r="P13" s="6"/>
       <c r="Q13" s="4"/>
@@ -2919,7 +3077,7 @@
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="N14" s="4">
         <v>1</v>
@@ -2928,7 +3086,7 @@
         <v>2</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
@@ -2950,12 +3108,12 @@
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="N15" s="6"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="6"/>
+      <c r="M15" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="N15" s="18"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="18"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
@@ -2977,7 +3135,7 @@
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="N16" s="4">
         <v>3</v>
@@ -2986,7 +3144,7 @@
         <v>3</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
@@ -3008,12 +3166,12 @@
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
-      <c r="M17" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="N17" s="6"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="6"/>
+      <c r="M17" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="18"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
@@ -3035,7 +3193,7 @@
       <c r="K18" s="4"/>
       <c r="L18" s="4"/>
       <c r="M18" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N18" s="4">
         <v>4</v>
@@ -3044,7 +3202,7 @@
         <v>4</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
@@ -3067,7 +3225,7 @@
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
       <c r="M19" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="N19" s="4">
         <v>4</v>
@@ -3076,7 +3234,7 @@
         <v>0</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
@@ -3098,12 +3256,12 @@
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4"/>
-      <c r="M20" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="N20" s="6"/>
-      <c r="O20" s="6"/>
-      <c r="P20" s="6"/>
+      <c r="M20" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="N20" s="18"/>
+      <c r="O20" s="18"/>
+      <c r="P20" s="18"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
@@ -3125,7 +3283,7 @@
       <c r="K21" s="4"/>
       <c r="L21" s="4"/>
       <c r="M21" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="N21" s="4">
         <v>0</v>
@@ -3134,7 +3292,7 @@
         <v>12</v>
       </c>
       <c r="P21" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
@@ -3156,10 +3314,12 @@
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
-      <c r="P22" s="4"/>
+      <c r="M22" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="N22" s="18"/>
+      <c r="O22" s="18"/>
+      <c r="P22" s="18"/>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
@@ -3180,10 +3340,14 @@
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
+      <c r="M23" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="N23" s="4"/>
       <c r="O23" s="4"/>
-      <c r="P23" s="4"/>
+      <c r="P23" s="4" t="s">
+        <v>59</v>
+      </c>
       <c r="Q23" s="4"/>
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
@@ -3191,14 +3355,30 @@
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
     </row>
+    <row r="24" spans="1:22">
+      <c r="M24" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="M15:P15"/>
+    <mergeCell ref="M17:P17"/>
+    <mergeCell ref="M20:P20"/>
+    <mergeCell ref="M22:P22"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:W12"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="4"/>
@@ -3259,10 +3439,10 @@
         <v>10</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
@@ -3302,7 +3482,7 @@
         <v>7</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="U2" s="1" t="s">
         <v>12</v>
@@ -3316,7 +3496,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C3" s="4">
         <v>3</v>
@@ -3342,14 +3522,14 @@
       <c r="J3" s="4">
         <v>5</v>
       </c>
-      <c r="M3" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="N3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="9" t="s">
+        <v>97</v>
+      </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="T3" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="U3" s="4">
         <v>12</v>
@@ -3363,7 +3543,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C4" s="4">
         <v>3</v>
@@ -3390,7 +3570,7 @@
         <v>4</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N4" s="4">
         <v>2</v>
@@ -3402,13 +3582,13 @@
         <v>17</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="U4" s="4">
         <v>7</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:23">
@@ -3416,7 +3596,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C5" s="4">
         <v>3</v>
@@ -3443,7 +3623,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="N5" s="4">
         <v>5</v>
@@ -3452,23 +3632,23 @@
         <v>0</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="U5" s="4">
         <v>3</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:23">
-      <c r="M6" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="N6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="9" t="s">
+        <v>96</v>
+      </c>
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
     </row>
@@ -3483,12 +3663,12 @@
         <v>0</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:23">
       <c r="M8" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N8" s="4">
         <v>1</v>
@@ -3497,16 +3677,16 @@
         <v>1</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:23">
-      <c r="M9" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
+      <c r="M9" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
     </row>
     <row r="10" spans="1:23">
       <c r="M10" s="4" t="s">
@@ -3519,20 +3699,20 @@
         <v>2</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:23">
-      <c r="M11" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
+      <c r="M11" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="N11" s="18"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="18"/>
     </row>
     <row r="12" spans="1:23">
       <c r="M12" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="N12" s="4">
         <v>4</v>
@@ -3541,17 +3721,45 @@
         <v>0</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23">
+      <c r="M13" s="6"/>
+      <c r="N13" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+    </row>
+    <row r="14" spans="1:23">
+      <c r="M14" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23">
+      <c r="M15" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="P15" s="4" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="M9:P9"/>
+    <mergeCell ref="M11:P11"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="27.33203125" customWidth="1"/>
@@ -3592,19 +3800,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C2" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" s="4">
         <v>0</v>
       </c>
       <c r="F2" s="4">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
@@ -3616,24 +3824,24 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C3" s="4">
+        <v>6</v>
+      </c>
+      <c r="D3" s="4">
         <v>5</v>
       </c>
-      <c r="D3" s="4">
-        <v>4</v>
-      </c>
       <c r="E3" s="4">
         <v>1</v>
       </c>
       <c r="F3" s="4">
-        <v>12</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="J3" s="6"/>
+        <v>14</v>
+      </c>
+      <c r="I3" s="16"/>
+      <c r="J3" s="9" t="s">
+        <v>98</v>
+      </c>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
     </row>
@@ -3642,31 +3850,31 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="4">
+        <v>6</v>
+      </c>
+      <c r="D4" s="4">
+        <v>4</v>
+      </c>
+      <c r="E4" s="4">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4">
+        <v>12</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
+        <v>3</v>
+      </c>
+      <c r="L4" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="C4" s="4">
-        <v>5</v>
-      </c>
-      <c r="D4" s="4">
-        <v>4</v>
-      </c>
-      <c r="E4" s="4">
-        <v>1</v>
-      </c>
-      <c r="F4" s="4">
-        <v>11</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="J4" s="4">
-        <v>0</v>
-      </c>
-      <c r="K4" s="4">
-        <v>3</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>75</v>
       </c>
       <c r="M4" s="4"/>
     </row>
@@ -3675,22 +3883,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C5" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" s="4">
         <v>3</v>
       </c>
       <c r="E5" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J5" s="4">
         <v>2</v>
@@ -3699,7 +3907,7 @@
         <v>1</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3707,22 +3915,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C6" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D6" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J6" s="4">
         <v>0</v>
@@ -3731,7 +3939,7 @@
         <v>3</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3739,7 +3947,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C7" s="4">
         <v>5</v>
@@ -3754,7 +3962,7 @@
         <v>3</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J7" s="4">
         <v>3</v>
@@ -3763,7 +3971,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -3771,7 +3979,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C8" s="4">
         <v>4</v>
@@ -3785,10 +3993,10 @@
       <c r="F8" s="4">
         <v>3</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="J8" s="6"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="9" t="s">
+        <v>99</v>
+      </c>
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
     </row>
@@ -3797,7 +4005,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C9" s="4">
         <v>5</v>
@@ -3812,7 +4020,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J9" s="4">
         <v>2</v>
@@ -3821,7 +4029,7 @@
         <v>1</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3829,22 +4037,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C10" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10" s="4">
         <v>0</v>
       </c>
       <c r="E10" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10" s="4">
         <v>0</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J10" s="4">
         <v>1</v>
@@ -3853,7 +4061,7 @@
         <v>2</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3864,7 +4072,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="I11" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J11" s="4">
         <v>0</v>
@@ -3873,47 +4081,37 @@
         <v>3</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="I12" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="J12" s="6"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="9" t="s">
+        <v>100</v>
+      </c>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
       <c r="I13" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="J13" s="4">
+        <v>2</v>
+      </c>
+      <c r="K13" s="4">
+        <v>1</v>
+      </c>
+      <c r="L13" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="J13" s="4">
-        <v>2</v>
-      </c>
-      <c r="K13" s="4">
-        <v>1</v>
-      </c>
-      <c r="L13" s="4" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="4"/>
       <c r="I14" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J14" s="4">
         <v>1</v>
@@ -3922,13 +4120,13 @@
         <v>2</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J15" s="4">
         <v>3</v>
@@ -3937,13 +4135,13 @@
         <v>0</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J16" s="4">
         <v>3</v>
@@ -3952,22 +4150,22 @@
         <v>0</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="4"/>
-      <c r="I17" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="J17" s="6"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="9" t="s">
+        <v>101</v>
+      </c>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="4"/>
       <c r="I18" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J18" s="4">
         <v>0</v>
@@ -3976,13 +4174,13 @@
         <v>3</v>
       </c>
       <c r="L18" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="4"/>
       <c r="I19" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="J19" s="4">
         <v>0</v>
@@ -3991,13 +4189,13 @@
         <v>3</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="4"/>
       <c r="I20" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J20" s="4">
         <v>3</v>
@@ -4006,22 +4204,22 @@
         <v>0</v>
       </c>
       <c r="L20" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="4"/>
-      <c r="I21" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
+      <c r="I21" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="4"/>
       <c r="I22" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J22" s="4">
         <v>3</v>
@@ -4030,26 +4228,26 @@
         <v>0</v>
       </c>
       <c r="L22" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="I23" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J23" s="4">
+        <v>3</v>
+      </c>
+      <c r="K23" s="4">
+        <v>0</v>
+      </c>
+      <c r="L23" s="4" t="s">
         <v>76</v>
-      </c>
-      <c r="J23" s="4">
-        <v>3</v>
-      </c>
-      <c r="K23" s="4">
-        <v>0</v>
-      </c>
-      <c r="L23" s="4" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:12">
       <c r="I24" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J24" s="4">
         <v>3</v>
@@ -4058,20 +4256,20 @@
         <v>0</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:12">
-      <c r="I25" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="6"/>
+      <c r="I25" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
     </row>
     <row r="26" spans="1:12">
       <c r="I26" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J26" s="4">
         <v>3</v>
@@ -4080,12 +4278,12 @@
         <v>0</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:12">
       <c r="I27" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J27" s="4">
         <v>1</v>
@@ -4094,12 +4292,12 @@
         <v>2</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:12">
       <c r="I28" s="4" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="J28" s="4">
         <v>0</v>
@@ -4108,12 +4306,12 @@
         <v>3</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:12">
       <c r="I29" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J29" s="4">
         <v>0</v>
@@ -4122,10 +4320,104 @@
         <v>3</v>
       </c>
       <c r="L29" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="I30" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="J30" s="17"/>
+      <c r="K30" s="17"/>
+      <c r="L30" s="17"/>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="I31" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="J31" s="4">
+        <v>0</v>
+      </c>
+      <c r="K31" s="4">
+        <v>3</v>
+      </c>
+      <c r="L31" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="I32" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J32" s="4">
+        <v>3</v>
+      </c>
+      <c r="K32" s="4">
+        <v>0</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33" spans="9:12">
+      <c r="I33" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J33" s="4">
+        <v>0</v>
+      </c>
+      <c r="K33" s="4">
+        <v>3</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="9:12">
+      <c r="I34" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="J34" s="17"/>
+      <c r="K34" s="17"/>
+      <c r="L34" s="17"/>
+    </row>
+    <row r="35" spans="9:12">
+      <c r="I35" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4"/>
+      <c r="L35" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="9:12">
+      <c r="I36" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="37" spans="9:12">
+      <c r="I37" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="I21:L21"/>
+    <mergeCell ref="I25:L25"/>
+    <mergeCell ref="I30:L30"/>
+    <mergeCell ref="I34:L34"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>